<commit_message>
Add consensus check: opex leverage, insurance-in-G&A test, valuation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7jWytf9AU1FJoCnFXNkUv
</commit_message>
<xml_diff>
--- a/model/VIA_software_services_mix.xlsx
+++ b/model/VIA_software_services_mix.xlsx
@@ -15,7 +15,8 @@
     <sheet name="Blended_Formula" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Contracts" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="ACV_CrossCheck" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Sources" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Consensus_Check" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Sources" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -119,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="491">
   <si>
     <t xml:space="preserve">VIA: software vs. services revenue mix</t>
   </si>
@@ -1168,6 +1169,162 @@
     <t xml:space="preserve">Sanity check vs benchmarks: TfL Dial-a-Ride software ~$0.59M/yr; LA Metro's Spare software $0.45M; Arlington software ~4% of $10.4M ≈ $0.4M.</t>
   </si>
   <si>
+    <t xml:space="preserve">What consensus already assumes (Bloomberg BST, user-provided file)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: model/Consensus_Projections_BBG.xlsx (Bloomberg, as provided). $mm. Q3'25–Q2'26 actual, Q3'26–Q4'27 consensus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q3'25A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4'25A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1'26A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2'26A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q3'26E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4'26E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q1'27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2'27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q3'27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4'27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total opex (GAAP, incl. SBC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  of which G&amp;A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock-based compensation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjusted EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance payables (BS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acquisitions, net of cash (CF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derived</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opex / revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adj. EBITDA margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue QoQ growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27E vs FY26E growth: revenue / opex / G&amp;A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test: can G&amp;A stay flat if insurance sits in G&amp;A?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance expense as % of revenue (Bleecker est. 3–4pts of GM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incremental insurance FY27E vs FY26E ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consensus total G&amp;A increase FY27E vs FY26E ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance growth as % of consensus G&amp;A growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer support costs also sit in G&amp;A (10-K) and scale with rides/hours; not quantified here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valuation at current price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share price ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stockanalysis.com, ~Sep 2026: mkt cap $2.41B / 81.51M shares. Update to the live price.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diluted shares (mm, consensus Q4'26E)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash, Q2'26 ($mm; no debt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enterprise value ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV / revenue FY26E | FY27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV / gross profit FY26E | FY27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV / adj. EBITDA FY27E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Illustrative sum-of-the-parts on FY27E gross profit (multiples are placeholders: source comps)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Services share of revenue (Bleecker_Replication updated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Services GM | software GM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY27E services GP | software GP ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV / GP multiple: services | software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholders. Justify with comps (outsourced transport operators vs vertical SaaS).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied EV ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied price per share ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upside / (downside) vs current</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blended EV/GP multiple the market pays today (FY27E)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software multiple needed to justify today's price, at services multiple above</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sources</t>
   </si>
   <si>
@@ -1418,6 +1575,21 @@
   </si>
   <si>
     <t xml:space="preserve">Colorado Politics: DougCo Feb 2026 $4.4M contract to continue/expand Link On Demand (Lone Tree, Highlands Ranch, Parker)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloomberg BST consensus projections (user-provided file, model/Consensus_Projections_BBG.xlsx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stockanalysis.com VIA statistics: mkt cap $2.41B, EV $2.09B, 81.51M shares, short interest 9.87% of float, 7.98 days to cover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://stockanalysis.com/stocks/via/statistics/</t>
   </si>
   <si>
     <t xml:space="preserve">User research notes (VIA_1.pdf): Arlington, DCTA, King County, Mobile, New Braunfels, Miami-Dade, Gastonia, Passaic, Q4'25 Texas example</t>
@@ -1427,7 +1599,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.0;&quot;($&quot;#,##0.0\);\-"/>
@@ -1436,6 +1608,9 @@
     <numFmt numFmtId="169" formatCode="\+0.0%;\-0.0%;0.0%"/>
     <numFmt numFmtId="170" formatCode="#,##0"/>
     <numFmt numFmtId="171" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="172" formatCode="#,##0.0"/>
+    <numFmt numFmtId="173" formatCode="0.0\x"/>
+    <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -1597,7 +1772,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1703,6 +1878,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6634,7 +6829,862 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:O46"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="3" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>357</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="O4" s="9" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>109.653</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>118.909</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>127.434</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>135.707</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>138</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>150.5556</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>156.6667</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>167.4444</v>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>169.1111</v>
+      </c>
+      <c r="L5" s="10" t="n">
+        <v>181.5556</v>
+      </c>
+      <c r="N5" s="11" t="n">
+        <f aca="false">SUM(E5:H5)</f>
+        <v>551.6966</v>
+      </c>
+      <c r="O5" s="11" t="n">
+        <f aca="false">SUM(I5:L5)</f>
+        <v>674.7778</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>43.086</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>46.953</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>50.055</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>55.606</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>54.7256</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>60.266</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>63.1311</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>68.0971</v>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>69.145</v>
+      </c>
+      <c r="L6" s="10" t="n">
+        <v>75.006</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <f aca="false">SUM(E6:H6)</f>
+        <v>220.6526</v>
+      </c>
+      <c r="O6" s="11" t="n">
+        <f aca="false">SUM(I6:L6)</f>
+        <v>275.3792</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>61.977</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>71.344</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>73.639</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>77.36</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>75.8772</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>76.1139</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>76.7026</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>78.2679</v>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v>78.3161</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>81.6391</v>
+      </c>
+      <c r="N7" s="11" t="n">
+        <f aca="false">SUM(E7:H7)</f>
+        <v>302.9901</v>
+      </c>
+      <c r="O7" s="11" t="n">
+        <f aca="false">SUM(I7:L7)</f>
+        <v>314.9257</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>21.189</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>27.615</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>28.621</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>30.11</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>29.1743</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>29.3484</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>29.3128</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>29.722</v>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>29.7493</v>
+      </c>
+      <c r="L8" s="10" t="n">
+        <v>30.5597</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <f aca="false">SUM(E8:H8)</f>
+        <v>117.2537</v>
+      </c>
+      <c r="O8" s="11" t="n">
+        <f aca="false">SUM(I8:L8)</f>
+        <v>119.3438</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>6.592</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>14.396</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>15.564</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>15.5808</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>16.1594</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>15.935</v>
+      </c>
+      <c r="J9" s="10" t="n">
+        <v>16.1104</v>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>16.2258</v>
+      </c>
+      <c r="L9" s="10" t="n">
+        <v>16.5433</v>
+      </c>
+      <c r="N9" s="11" t="n">
+        <f aca="false">SUM(E9:H9)</f>
+        <v>63.3142</v>
+      </c>
+      <c r="O9" s="11" t="n">
+        <f aca="false">SUM(I9:L9)</f>
+        <v>64.8145</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>-8.692</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>-7.384</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>-5.809</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>-0.003441</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>-4.0322</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>2.4098</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>3.4154</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>6.9811</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>7.79</v>
+      </c>
+      <c r="L10" s="10" t="n">
+        <v>11.2567</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <f aca="false">SUM(E10:H10)</f>
+        <v>-7.434841</v>
+      </c>
+      <c r="O10" s="11" t="n">
+        <f aca="false">SUM(I10:L10)</f>
+        <v>29.4432</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>15.751</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>15.144</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>14.882</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>15.329</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>14.9242</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>18.1774</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>18.3044</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>20.1841</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>20.0667</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>22.0113</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>-39.892</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>-7.515</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>-14.157</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>-15</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>-15</v>
+      </c>
+      <c r="K12" s="10" t="n">
+        <v>-7.505</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <v>-16.3677</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <f aca="false">SUM(E12:H12)</f>
+        <v>-21.393</v>
+      </c>
+      <c r="O12" s="11" t="n">
+        <f aca="false">SUM(I12:L12)</f>
+        <v>-53.8727</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="3" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <f aca="false">C6/C5</f>
+        <v>0.392930425980137</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <f aca="false">D6/D5</f>
+        <v>0.394864980783625</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <f aca="false">E6/E5</f>
+        <v>0.392791562691275</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <f aca="false">F6/F5</f>
+        <v>0.409750418180344</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <f aca="false">G6/G5</f>
+        <v>0.39656231884058</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <f aca="false">H6/H5</f>
+        <v>0.400290656740766</v>
+      </c>
+      <c r="I15" s="15" t="n">
+        <f aca="false">I6/I5</f>
+        <v>0.402964382348004</v>
+      </c>
+      <c r="J15" s="15" t="n">
+        <f aca="false">J6/J5</f>
+        <v>0.406684845835394</v>
+      </c>
+      <c r="K15" s="15" t="n">
+        <f aca="false">K6/K5</f>
+        <v>0.408873220031092</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <f aca="false">L6/L5</f>
+        <v>0.413129641828729</v>
+      </c>
+      <c r="N15" s="15" t="n">
+        <f aca="false">N6/N5</f>
+        <v>0.399952800144137</v>
+      </c>
+      <c r="O15" s="15" t="n">
+        <f aca="false">O6/O5</f>
+        <v>0.408103526820236</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <f aca="false">C7/C5</f>
+        <v>0.565210254165413</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <f aca="false">D7/D5</f>
+        <v>0.599988226290693</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <f aca="false">E7/E5</f>
+        <v>0.577859911797479</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <f aca="false">F7/F5</f>
+        <v>0.570051655404659</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <f aca="false">G7/G5</f>
+        <v>0.549834782608696</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <f aca="false">H7/H5</f>
+        <v>0.505553430094928</v>
+      </c>
+      <c r="I16" s="15" t="n">
+        <f aca="false">I7/I5</f>
+        <v>0.489590959661498</v>
+      </c>
+      <c r="J16" s="15" t="n">
+        <f aca="false">J7/J5</f>
+        <v>0.467426202369264</v>
+      </c>
+      <c r="K16" s="15" t="n">
+        <f aca="false">K7/K5</f>
+        <v>0.463104432529858</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <f aca="false">L7/L5</f>
+        <v>0.449664455406498</v>
+      </c>
+      <c r="N16" s="15" t="n">
+        <f aca="false">N7/N5</f>
+        <v>0.549196968043668</v>
+      </c>
+      <c r="O16" s="15" t="n">
+        <f aca="false">O7/O5</f>
+        <v>0.466710226684992</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="C17" s="15" t="n">
+        <f aca="false">C10/C5</f>
+        <v>-0.079268237075137</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <f aca="false">D10/D5</f>
+        <v>-0.062097906802681</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <f aca="false">E10/E5</f>
+        <v>-0.0455843809344445</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <f aca="false">F10/F5</f>
+        <v>-2.53560980642119E-005</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <f aca="false">G10/G5</f>
+        <v>-0.0292188405797101</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <f aca="false">H10/H5</f>
+        <v>0.0160060469354843</v>
+      </c>
+      <c r="I17" s="15" t="n">
+        <f aca="false">I10/I5</f>
+        <v>0.0218004208935275</v>
+      </c>
+      <c r="J17" s="15" t="n">
+        <f aca="false">J10/J5</f>
+        <v>0.0416920482261575</v>
+      </c>
+      <c r="K17" s="15" t="n">
+        <f aca="false">K10/K5</f>
+        <v>0.046064391988462</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <f aca="false">L10/L5</f>
+        <v>0.0620013924109199</v>
+      </c>
+      <c r="N17" s="15" t="n">
+        <f aca="false">N10/N5</f>
+        <v>-0.0134763219494193</v>
+      </c>
+      <c r="O17" s="15" t="n">
+        <f aca="false">O10/O5</f>
+        <v>0.0436339191953262</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <f aca="false">D5/C5-1</f>
+        <v>0.0844117352010434</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <f aca="false">E5/D5-1</f>
+        <v>0.0716934798879816</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <f aca="false">F5/E5-1</f>
+        <v>0.0649198800947941</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <f aca="false">G5/F5-1</f>
+        <v>0.0168966965594997</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <f aca="false">H5/G5-1</f>
+        <v>0.0909826086956522</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <f aca="false">I5/H5-1</f>
+        <v>0.0405903201209388</v>
+      </c>
+      <c r="J18" s="15" t="n">
+        <f aca="false">J5/I5-1</f>
+        <v>0.0687938151502521</v>
+      </c>
+      <c r="K18" s="15" t="n">
+        <f aca="false">K5/J5-1</f>
+        <v>0.00995375181254188</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <f aca="false">L5/K5-1</f>
+        <v>0.0735877183697582</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="C19" s="15" t="n">
+        <f aca="false">O5/N5-1</f>
+        <v>0.22309581026963</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <f aca="false">O7/N7-1</f>
+        <v>0.0393927062303356</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <f aca="false">O8/N8-1</f>
+        <v>0.0178254502842981</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="3" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <f aca="false">C22*(O5-N5)</f>
+        <v>4.307842</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <f aca="false">O8-N8</f>
+        <v>2.09009999999999</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="16" t="s">
+        <v>379</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <f aca="false">IF(C24=0,0,C23/C24)</f>
+        <v>2.06106980527248</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="18" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="3" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="C29" s="27" t="n">
+        <v>29.57</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C30" s="28" t="n">
+        <v>84.2146</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="16" t="s">
+        <v>386</v>
+      </c>
+      <c r="C32" s="11" t="n">
+        <f aca="false">C29*C30-C31</f>
+        <v>2154.225722</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="C33" s="29" t="n">
+        <f aca="false">C32/N5</f>
+        <v>3.90472901591201</v>
+      </c>
+      <c r="D33" s="29" t="n">
+        <f aca="false">C32/O5</f>
+        <v>3.19249643660476</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="C34" s="29" t="n">
+        <f aca="false">C32/N6</f>
+        <v>9.76297456726094</v>
+      </c>
+      <c r="D34" s="29" t="n">
+        <f aca="false">C32/O6</f>
+        <v>7.82276120346054</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="C35" s="29" t="n">
+        <f aca="false">C32/O10</f>
+        <v>73.1654752880122</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="3" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <f aca="false">Bleecker_Replication!E22</f>
+        <v>0.760412444588375</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <f aca="false">Bleecker_Replication!E19</f>
+        <v>0.292987009709526</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <f aca="false">Bleecker_Replication!E20</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="C40" s="11" t="n">
+        <f aca="false">O6*(C38*C39)/(C38*C39+(1-C38)*D39)</f>
+        <v>152.434280976514</v>
+      </c>
+      <c r="D40" s="11" t="n">
+        <f aca="false">O6-C40</f>
+        <v>122.944919023486</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="C41" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="C42" s="11" t="n">
+        <f aca="false">C40*C41+D40*D41</f>
+        <v>1686.7520331644</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="16" t="s">
+        <v>397</v>
+      </c>
+      <c r="C43" s="26" t="n">
+        <f aca="false">(C42+C31)/C30</f>
+        <v>24.0190184738086</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="16" t="s">
+        <v>398</v>
+      </c>
+      <c r="C44" s="31" t="n">
+        <f aca="false">C43/C29-1</f>
+        <v>-0.187723419891492</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="C45" s="29" t="n">
+        <f aca="false">C32/O6</f>
+        <v>7.82276120346054</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="C46" s="29" t="n">
+        <f aca="false">(C32-C40*C41)/D40</f>
+        <v>13.8023018157123</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -6644,100 +7694,100 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>349</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>350</v>
+      <c r="A2" s="32" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>351</v>
+        <v>403</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>352</v>
+        <v>404</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>353</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>354</v>
+        <v>406</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>355</v>
+        <v>407</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>356</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>357</v>
+        <v>409</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>358</v>
+        <v>410</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>359</v>
+        <v>411</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>360</v>
+        <v>412</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>361</v>
+        <v>413</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>362</v>
+        <v>414</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>363</v>
+        <v>415</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>364</v>
+        <v>416</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>365</v>
+        <v>417</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>366</v>
+        <v>418</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>367</v>
+        <v>419</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>368</v>
+        <v>420</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>369</v>
+        <v>421</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>370</v>
+        <v>422</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>371</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>372</v>
+        <v>424</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>373</v>
+        <v>425</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>374</v>
+        <v>426</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6745,43 +7795,43 @@
         <v>231</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>375</v>
+        <v>427</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>376</v>
+        <v>428</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>377</v>
+        <v>429</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>378</v>
+        <v>430</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>379</v>
+        <v>431</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>380</v>
+        <v>432</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>381</v>
+        <v>433</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>382</v>
+        <v>434</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>383</v>
+        <v>435</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>384</v>
+        <v>436</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>385</v>
+        <v>437</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6789,10 +7839,10 @@
         <v>258</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>386</v>
+        <v>438</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>387</v>
+        <v>439</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6800,21 +7850,21 @@
         <v>268</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>388</v>
+        <v>440</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>389</v>
+        <v>441</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>390</v>
+        <v>442</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>391</v>
+        <v>443</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>392</v>
+        <v>444</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6822,10 +7872,10 @@
         <v>262</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>393</v>
+        <v>445</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>394</v>
+        <v>446</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6833,21 +7883,21 @@
         <v>281</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>395</v>
+        <v>447</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>396</v>
+        <v>448</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>397</v>
+        <v>449</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>398</v>
+        <v>450</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>399</v>
+        <v>451</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6855,10 +7905,10 @@
         <v>289</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>400</v>
+        <v>452</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>401</v>
+        <v>453</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6866,10 +7916,10 @@
         <v>294</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>402</v>
+        <v>454</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>403</v>
+        <v>455</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6877,21 +7927,21 @@
         <v>245</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>404</v>
+        <v>456</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>405</v>
+        <v>457</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>406</v>
+        <v>458</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>407</v>
+        <v>459</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>408</v>
+        <v>460</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6899,10 +7949,10 @@
         <v>299</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>409</v>
+        <v>461</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>410</v>
+        <v>462</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6910,21 +7960,21 @@
         <v>221</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>411</v>
+        <v>463</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>412</v>
+        <v>464</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>413</v>
+        <v>465</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>414</v>
+        <v>466</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>415</v>
+        <v>467</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6932,10 +7982,10 @@
         <v>239</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>416</v>
+        <v>468</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>417</v>
+        <v>469</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6943,65 +7993,65 @@
         <v>277</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>418</v>
+        <v>470</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>419</v>
+        <v>471</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>420</v>
+        <v>472</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>421</v>
+        <v>473</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>422</v>
+        <v>474</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>423</v>
+        <v>475</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>424</v>
+        <v>476</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>362</v>
+        <v>414</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>425</v>
+        <v>477</v>
       </c>
       <c r="B33" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>426</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>427</v>
+        <v>479</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>428</v>
+        <v>480</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>429</v>
+        <v>481</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>430</v>
+        <v>482</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>431</v>
+        <v>483</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>376</v>
+        <v>428</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7009,20 +8059,40 @@
         <v>254</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>432</v>
+        <v>484</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>399</v>
+        <v>451</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="C37" s="4"/>
+      <c r="B39" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="C39" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Add Bloomberg comps sheet; update price to $28.37
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7jWytf9AU1FJoCnFXNkUv
</commit_message>
<xml_diff>
--- a/model/VIA_software_services_mix.xlsx
+++ b/model/VIA_software_services_mix.xlsx
@@ -16,7 +16,8 @@
     <sheet name="Contracts" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="ACV_CrossCheck" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Consensus_Check" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="Sources" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Comps_BBG" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Sources" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -120,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="522">
   <si>
     <t xml:space="preserve">VIA: software vs. services revenue mix</t>
   </si>
@@ -1271,10 +1272,10 @@
     <t xml:space="preserve">Share price ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">stockanalysis.com, ~Sep 2026: mkt cap $2.41B / 81.51M shares. Update to the live price.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diluted shares (mm, consensus Q4'26E)</t>
+    <t xml:space="preserve">Bloomberg, Sep 2026 close (user screenshot). BBG: mkt cap $2.31B, EV $1.99B.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shares outstanding (mm, basic; ties to BBG mkt cap)</t>
   </si>
   <si>
     <t xml:space="preserve">Cash, Q2'26 ($mm; no debt)</t>
@@ -1325,6 +1326,93 @@
     <t xml:space="preserve">Software multiple needed to justify today's price, at services multiple above</t>
   </si>
   <si>
+    <t xml:space="preserve">Bloomberg RV: 'BICS Best Fit' comps (VIA classified 100% Application Software)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: Bloomberg RV screen, user screenshot, price $28.37 (Sep 2026). '--' = not meaningful (negative). FY1 = 2026, FY2 = 2027.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mkt cap ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV/EBITDA LTM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV/EBITDA FY1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV/EBITDA FY2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/E FY1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/E FY2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/FCF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LiveRamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethos Technologies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DoubleVerify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privia Health</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutron Holdings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertex Inc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACV Auctions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pagaya Technologies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SoundHound AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Progress Software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comp median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIA (Bloomberg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIA premium to median (x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blended forward P/E (chart): VIA 96.6x vs comps avg 30.6x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Bloomberg's own classification puts VIA 100% in Application Software. Screens and quant peer sets benchmark it against software, even though ~75% of revenue is services.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• These 'peers' are a grab-bag (ad-tech, health services, auctions, fintech). Use this to show how the market labels VIA, not as the valuation comp set.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• EV/EBITDA on near-breakeven EBITDA exaggerates the premium. Anchor valuation on EV/GP and EV/Sales (Consensus_Check) with separate software and services comp sets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• The chart shows VIA's forward P/E expanding from ~50x to ~97x from late July into September, around the Q2 print (Aug 6), while comps held ~30x. Mgmt says the Q2 margin beat came from one-time revenue that will revert.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sources</t>
   </si>
   <si>
@@ -1590,6 +1678,12 @@
   </si>
   <si>
     <t xml:space="preserve">https://stockanalysis.com/stocks/via/statistics/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloomberg RV screen (BICS Best Fit comps), user screenshot, Sep 2026</t>
   </si>
   <si>
     <t xml:space="preserve">User research notes (VIA_1.pdf): Arlington, DCTA, King County, Mobile, New Braunfels, Miami-Dade, Gastonia, Passaic, Q4'25 Texas example</t>
@@ -1599,7 +1693,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.0;&quot;($&quot;#,##0.0\);\-"/>
@@ -1611,6 +1705,7 @@
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
     <numFmt numFmtId="173" formatCode="0.0\x"/>
     <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%"/>
+    <numFmt numFmtId="175" formatCode="0.00"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -1772,7 +1867,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1898,6 +1993,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2402,6 +2505,441 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C40"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="100"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="34" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>458</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>465</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="C39" s="4"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="C40" s="4"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -7503,7 +8041,7 @@
         <v>382</v>
       </c>
       <c r="C29" s="27" t="n">
-        <v>29.57</v>
+        <v>28.37</v>
       </c>
       <c r="D29" s="18" t="s">
         <v>383</v>
@@ -7514,7 +8052,7 @@
         <v>384</v>
       </c>
       <c r="C30" s="28" t="n">
-        <v>84.2146</v>
+        <v>81.51</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7531,7 +8069,7 @@
       </c>
       <c r="C32" s="11" t="n">
         <f aca="false">C29*C30-C31</f>
-        <v>2154.225722</v>
+        <v>1976.4387</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7540,11 +8078,11 @@
       </c>
       <c r="C33" s="29" t="n">
         <f aca="false">C32/N5</f>
-        <v>3.90472901591201</v>
+        <v>3.58247395398123</v>
       </c>
       <c r="D33" s="29" t="n">
         <f aca="false">C32/O5</f>
-        <v>3.19249643660476</v>
+        <v>2.92902152382607</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7553,11 +8091,11 @@
       </c>
       <c r="C34" s="29" t="n">
         <f aca="false">C32/N6</f>
-        <v>9.76297456726094</v>
+        <v>8.95724183626207</v>
       </c>
       <c r="D34" s="29" t="n">
         <f aca="false">C32/O6</f>
-        <v>7.82276120346054</v>
+        <v>7.17715317642001</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7566,7 +8104,7 @@
       </c>
       <c r="C35" s="29" t="n">
         <f aca="false">C32/O10</f>
-        <v>73.1654752880122</v>
+        <v>67.1271702804043</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7638,7 +8176,7 @@
       </c>
       <c r="C43" s="26" t="n">
         <f aca="false">(C42+C31)/C30</f>
-        <v>24.0190184738086</v>
+        <v>24.8159984439259</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7647,7 +8185,7 @@
       </c>
       <c r="C44" s="31" t="n">
         <f aca="false">C43/C29-1</f>
-        <v>-0.187723419891492</v>
+        <v>-0.125273230739306</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7656,7 +8194,7 @@
       </c>
       <c r="C45" s="29" t="n">
         <f aca="false">C32/O6</f>
-        <v>7.82276120346054</v>
+        <v>7.17715317642001</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7665,7 +8203,7 @@
       </c>
       <c r="C46" s="29" t="n">
         <f aca="false">(C32-C40*C41)/D40</f>
-        <v>13.8023018157123</v>
+        <v>12.356231303713</v>
       </c>
     </row>
   </sheetData>
@@ -7684,417 +8222,444 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="80"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="3" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="B1" s="1" t="s">
         <v>401</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="32" t="s">
+      <c r="B2" s="2" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9" t="s">
         <v>403</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>404</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>405</v>
       </c>
+      <c r="E4" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>409</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>411</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>406</v>
-      </c>
       <c r="B5" s="4" t="s">
-        <v>407</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>408</v>
+        <v>412</v>
+      </c>
+      <c r="C5" s="32" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="D5" s="32" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="G5" s="32" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="H5" s="32" t="n">
+        <v>13.06</v>
+      </c>
+      <c r="I5" s="32" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="J5" s="32" t="n">
+        <v>11.96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>409</v>
-      </c>
       <c r="B6" s="4" t="s">
-        <v>410</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
+      </c>
+      <c r="C6" s="32" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="D6" s="32" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="F6" s="32" t="n">
+        <v>17.58</v>
+      </c>
+      <c r="G6" s="32" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="I6" s="32" t="n">
+        <v>22.86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>412</v>
-      </c>
       <c r="B7" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="C7" s="4" t="s">
         <v>414</v>
       </c>
+      <c r="C7" s="32" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="D7" s="32" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="F7" s="32" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="G7" s="32" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="H7" s="32" t="n">
+        <v>27.18</v>
+      </c>
+      <c r="I7" s="32" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="J7" s="32" t="n">
+        <v>13.22</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="B8" s="4" t="s">
         <v>415</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="32" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="D8" s="32" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>37.55</v>
+      </c>
+      <c r="F8" s="32" t="n">
+        <v>14.03</v>
+      </c>
+      <c r="G8" s="32" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="H8" s="32" t="n">
+        <v>27.56</v>
+      </c>
+      <c r="I8" s="32" t="n">
+        <v>21.87</v>
+      </c>
+      <c r="J8" s="32" t="n">
+        <v>18.21</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="s">
         <v>416</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C9" s="32" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="D9" s="32" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="F9" s="32" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="G9" s="32" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="H9" s="32" t="n">
+        <v>6.79</v>
+      </c>
+      <c r="I9" s="32" t="n">
+        <v>21.39</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="4" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="C10" s="32" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="D10" s="32" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>17.67</v>
+      </c>
+      <c r="F10" s="32" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="H10" s="32" t="n">
+        <v>14.38</v>
+      </c>
+      <c r="I10" s="32" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="J10" s="32" t="n">
+        <v>26.35</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="4" t="s">
         <v>418</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C11" s="32" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="D11" s="32" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="E11" s="32" t="n">
+        <v>123.93</v>
+      </c>
+      <c r="F11" s="32" t="n">
+        <v>23.14</v>
+      </c>
+      <c r="G11" s="32" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="H11" s="32" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="I11" s="32" t="n">
+        <v>57.42</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
         <v>419</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C12" s="32" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="D12" s="32" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="E12" s="32" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="F12" s="32" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G12" s="32" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="H12" s="32" t="n">
+        <v>6.62</v>
+      </c>
+      <c r="I12" s="32" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="J12" s="32" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="C13" s="32" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D13" s="32" t="n">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C14" s="32" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="D14" s="32" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="E14" s="32" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="F14" s="32" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="G14" s="32" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="H14" s="32" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="I14" s="32" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="J14" s="32" t="n">
+        <v>5.64</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="16" t="s">
         <v>422</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C15" s="33" t="n">
+        <f aca="false">MEDIAN(C5:C14)</f>
+        <v>1.995</v>
+      </c>
+      <c r="D15" s="33" t="n">
+        <f aca="false">MEDIAN(D5:D14)</f>
+        <v>2.085</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <f aca="false">MEDIAN(E5:E14)</f>
+        <v>15.17</v>
+      </c>
+      <c r="F15" s="33" t="n">
+        <f aca="false">MEDIAN(F5:F14)</f>
+        <v>8.48</v>
+      </c>
+      <c r="G15" s="33" t="n">
+        <f aca="false">MEDIAN(G5:G14)</f>
+        <v>7.16</v>
+      </c>
+      <c r="H15" s="33" t="n">
+        <f aca="false">MEDIAN(H5:H14)</f>
+        <v>13.72</v>
+      </c>
+      <c r="I15" s="33" t="n">
+        <f aca="false">MEDIAN(I5:I14)</f>
+        <v>21.14</v>
+      </c>
+      <c r="J15" s="33" t="n">
+        <f aca="false">MEDIAN(J5:J14)</f>
+        <v>12.59</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="16" t="s">
         <v>423</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="C16" s="32" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="G16" s="32" t="n">
+        <v>69.64</v>
+      </c>
+      <c r="I16" s="32" t="n">
+        <v>67.87</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="16" t="s">
         <v>424</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="G17" s="29" t="n">
+        <f aca="false">G16/G15</f>
+        <v>9.72625698324022</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <f aca="false">I16/I15</f>
+        <v>3.21050141911069</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="18" t="s">
         <v>425</v>
       </c>
-      <c r="C11" s="4" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="7" t="s">
         <v>426</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B12" s="4" t="s">
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="7" t="s">
         <v>427</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="7" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>440</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>443</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>445</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>447</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>449</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>450</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>289</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>452</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>454</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>456</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>458</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>459</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>461</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>463</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>465</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>466</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>239</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>470</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>472</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>475</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>476</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>478</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>479</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>480</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>482</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>483</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>484</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>485</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>486</v>
-      </c>
-      <c r="C37" s="4"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>487</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>488</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>490</v>
-      </c>
-      <c r="C39" s="4"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B22:J22"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="B24:J24"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Add stream-based revenue build and DCF with short/bull scenarios
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7jWytf9AU1FJoCnFXNkUv
</commit_message>
<xml_diff>
--- a/model/VIA_software_services_mix.xlsx
+++ b/model/VIA_software_services_mix.xlsx
@@ -17,7 +17,9 @@
     <sheet name="ACV_CrossCheck" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Consensus_Check" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Comps_BBG" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="Sources" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Revenue_Build" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="DCF" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Sources" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -121,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="669">
   <si>
     <t xml:space="preserve">VIA: software vs. services revenue mix</t>
   </si>
@@ -1411,6 +1413,447 @@
   </si>
   <si>
     <t xml:space="preserve">• The chart shows VIA's forward P/E expanding from ~50x to ~97x from late July into September, around the Q2 print (Aug 6), while comps held ~30x. Mgmt says the Q2 margin beat came from one-time revenue that will revert.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue build and operating model by revenue stream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Four streams with different economics: software, microtransit/paratransit services (hours × $/hr), network deals (contract value launched), one-time. FY25 actual; FY26 matched to consensus; FY27–30 driven by inputs; FY31–35 growth fades linearly to terminal growth.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO: 1 = Short case, 2 = Bull (matches consensus FY26–27)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY28E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY29E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY30E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY31E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY32E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY33E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY34E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY35E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consensus revenue (BBG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consensus adj. EBITDA (BBG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25A from company (adj. EBITDA ≈ −$32M); FY26–27 Bloomberg consensus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRIVERS (Short / Bull input rows; 'Live' row feeds the model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software revenue growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 incl. Downtowner. Software ≈ customers × revenue per customer; organic customer growth ~9%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Short</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Bull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Live</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours: expansion at existing customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-K: expansion with existing customers drives most growth.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours: new customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organic logo growth ~9% but new logos start small.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours: downsell / budget cuts / churn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short: funding tightens 2027 (stopgap, ARPA end). Jersey City −50%, Arlington −31%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price escalator ($/hr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3% annual escalator in Via's Q4'25 example contract.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Network: contract value launched ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 wins &gt;$40M + Rochester $14.6M, mostly launching H2'26–27. ~$10–15M per deal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Network: rebid loss (% of opening run-rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5-yr terms: first rebids ~2029 (Sioux Falls through 2028).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time revenue (% of total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3% in FY24 and FY25 (10-K).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software gross margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bleecker assumption; reported cost split implies ~73%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microtransit/paratransit gross margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bleecker_Replication updated TaaS GM. Bull: +1pt/yr from AI/routing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Network gross margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSUMPTION (undisclosed). Short: bus-operator economics. CFO: 'some accretive, some less.'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time gross margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-margin implementation/consulting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hour-driven opex (% of services revenue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance (~3.5%, Bleecker) + customer support (~3%, Bleecker unit economics), both in G&amp;A (10-K). Bull: AI cuts support.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed opex growth (R&amp;D, S&amp;M, corporate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consensus total opex +3.9% FY27.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminal growth (from DCF tab)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Network opening run-rate FY26 ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate: Mobile $12.1M + Sioux Falls + Twin Cities (MI). Sioux Falls value/structure unverified.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blended $/vehicle-hour FY25 (for implied hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Illustrative: 2026 rates $64.5–70 micro, $67.75 para; legacy lower ($42–50).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVENUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25 est: 24% of recurring revenue (services ~76%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microtransit / paratransit services (hours × $/hr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25–26: residual so total = actual/consensus. FY27+: hours growth (expansion + new − cuts) × price escalator.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue = opening run-rate (escalated, net of rebid losses) + half of the year's launches.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recurring subtotal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time (implementation, consulting)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL REVENUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   vs consensus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Services share (micro/para + network)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Blended $/vehicle-hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Implied micro/para vehicle-hours (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Network detail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Opening run-rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Opening after escalator and rebid losses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Launched in year (links driver)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Closing run-rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROSS PROFIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Microtransit / paratransit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Network</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL GROSS PROFIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Gross margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Consensus gross margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPERATING COSTS (adjusted: ex-SBC, ex-D&amp;A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hour-driven (insurance, support): % × services revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed (R&amp;D, S&amp;M, corporate); FY26 matched to consensus EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 backed out so adj. EBITDA = consensus (−$7.4M).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total adjusted opex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   % of revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADJUSTED EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjusted = before stock comp. DCF tab deducts stock comp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   vs consensus ($mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DCF (unlevered free cash flow, valuation at end-FY26, mid-year convention)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario is set on Revenue_Build!D4. Stock comp is deducted as a real cost (toggle below).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk-free rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-yr UST (update).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small-cap, high-growth; check Bloomberg BETA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity risk premium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost of equity = WACC (no debt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via has no debt (10-Q).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WACC used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Override here to test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminal growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash tax rate (after NOLs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First year of cash taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOL shield assumption. Check 10-K tax note.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D&amp;A % of revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consensus D&amp;A ≈ $9–10M on ~$550M.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capex + capitalized software % of revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY25 capitalized software $4.3M + capex.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net working capital % of revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q2'26: AR+prepaids ≈ $122M less payables/accruals/deferred ≈ $81M → ~$41M on $543M run-rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deduct stock comp? (1 = yes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SBC is ~11% of revenue in FY26.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash (Q2'26, no debt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diluted shares (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consensus Q4'26E diluted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current share price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exit EV/EBITDA multiple (cross-check)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied to FY35 adj. EBITDA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock comp % of revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26–27 = consensus SBC; fades to 5%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock comp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA after stock comp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D&amp;A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capex + capitalized software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increase in net working capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FY26 excluded (valuation at end-FY26).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNLEVERED FREE CASH FLOW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discount period (years from end-FY26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PV of FCF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALUATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum of PV of FCF (FY27–35)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminal value (perpetuity growth) at end-FY35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PV of terminal value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enterprise value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Cash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALUE PER SHARE (perpetuity growth)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upside / (downside) vs current price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminal value as % of EV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-check: exit multiple on FY35 adj. EBITDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Value per share (exit multiple)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Implied perpetuity growth in exit multiple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensitivity: value per share (perpetuity), WACC (rows) × terminal growth (cols)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WACC \ g</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario results (switch Revenue_Build!D4 to 1 or 2 and re-read C43). Our run is recorded in the README.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>
@@ -1693,7 +2136,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.0;&quot;($&quot;#,##0.0\);\-"/>
@@ -1706,6 +2149,7 @@
     <numFmt numFmtId="173" formatCode="0.0\x"/>
     <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%"/>
     <numFmt numFmtId="175" formatCode="0.00"/>
+    <numFmt numFmtId="176" formatCode="0.0"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -1867,7 +2311,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2001,6 +2445,34 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="175" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2510,6 +2982,3695 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:N107"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="16" t="s">
+        <v>432</v>
+      </c>
+      <c r="D4" s="34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>434</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="M6" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="N6" s="9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>434.337</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>551.697</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>674.778</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>-32.4</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>-7.435</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>29.443</v>
+      </c>
+      <c r="N8" s="18" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <f aca="false">IF($D$4=1,D12,D13)</f>
+        <v>0.18</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <f aca="false">IF($D$4=1,E12,E13)</f>
+        <v>0.12</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <f aca="false">IF($D$4=1,F12,F13)</f>
+        <v>0.11</v>
+      </c>
+      <c r="G14" s="15" t="n">
+        <f aca="false">IF($D$4=1,G12,G13)</f>
+        <v>0.1</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <f aca="false">IF($D$4=1,H12,H13)</f>
+        <v>0.09</v>
+      </c>
+      <c r="I14" s="15" t="n">
+        <f aca="false">$H14</f>
+        <v>0.09</v>
+      </c>
+      <c r="J14" s="15" t="n">
+        <f aca="false">$H14</f>
+        <v>0.09</v>
+      </c>
+      <c r="K14" s="15" t="n">
+        <f aca="false">$H14</f>
+        <v>0.09</v>
+      </c>
+      <c r="L14" s="15" t="n">
+        <f aca="false">$H14</f>
+        <v>0.09</v>
+      </c>
+      <c r="M14" s="15" t="n">
+        <f aca="false">$H14</f>
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="16" t="s">
+        <v>452</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <f aca="false">IF($D$4=1,E16,E17)</f>
+        <v>0.12</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <f aca="false">IF($D$4=1,F16,F17)</f>
+        <v>0.11</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <f aca="false">IF($D$4=1,G16,G17)</f>
+        <v>0.1</v>
+      </c>
+      <c r="H18" s="15" t="n">
+        <f aca="false">IF($D$4=1,H16,H17)</f>
+        <v>0.1</v>
+      </c>
+      <c r="I18" s="15" t="n">
+        <f aca="false">$H18</f>
+        <v>0.1</v>
+      </c>
+      <c r="J18" s="15" t="n">
+        <f aca="false">$H18</f>
+        <v>0.1</v>
+      </c>
+      <c r="K18" s="15" t="n">
+        <f aca="false">$H18</f>
+        <v>0.1</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <f aca="false">$H18</f>
+        <v>0.1</v>
+      </c>
+      <c r="M18" s="15" t="n">
+        <f aca="false">$H18</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="16" t="s">
+        <v>454</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H21" s="13" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <f aca="false">IF($D$4=1,E20,E21)</f>
+        <v>0.04</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <f aca="false">IF($D$4=1,F20,F21)</f>
+        <v>0.04</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <f aca="false">IF($D$4=1,G20,G21)</f>
+        <v>0.04</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <f aca="false">IF($D$4=1,H20,H21)</f>
+        <v>0.04</v>
+      </c>
+      <c r="I22" s="15" t="n">
+        <f aca="false">$H22</f>
+        <v>0.04</v>
+      </c>
+      <c r="J22" s="15" t="n">
+        <f aca="false">$H22</f>
+        <v>0.04</v>
+      </c>
+      <c r="K22" s="15" t="n">
+        <f aca="false">$H22</f>
+        <v>0.04</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <f aca="false">$H22</f>
+        <v>0.04</v>
+      </c>
+      <c r="M22" s="15" t="n">
+        <f aca="false">$H22</f>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="16" t="s">
+        <v>456</v>
+      </c>
+      <c r="N23" s="6" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>-0.07</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="H24" s="13" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="H25" s="13" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="E26" s="15" t="n">
+        <f aca="false">IF($D$4=1,E24,E25)</f>
+        <v>-0.08</v>
+      </c>
+      <c r="F26" s="15" t="n">
+        <f aca="false">IF($D$4=1,F24,F25)</f>
+        <v>-0.07</v>
+      </c>
+      <c r="G26" s="15" t="n">
+        <f aca="false">IF($D$4=1,G24,G25)</f>
+        <v>-0.06</v>
+      </c>
+      <c r="H26" s="15" t="n">
+        <f aca="false">IF($D$4=1,H24,H25)</f>
+        <v>-0.06</v>
+      </c>
+      <c r="I26" s="15" t="n">
+        <f aca="false">$H26</f>
+        <v>-0.06</v>
+      </c>
+      <c r="J26" s="15" t="n">
+        <f aca="false">$H26</f>
+        <v>-0.06</v>
+      </c>
+      <c r="K26" s="15" t="n">
+        <f aca="false">$H26</f>
+        <v>-0.06</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <f aca="false">$H26</f>
+        <v>-0.06</v>
+      </c>
+      <c r="M26" s="15" t="n">
+        <f aca="false">$H26</f>
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="16" t="s">
+        <v>458</v>
+      </c>
+      <c r="N27" s="6" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H28" s="13" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H29" s="13" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <f aca="false">IF($D$4=1,E28,E29)</f>
+        <v>0.03</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <f aca="false">IF($D$4=1,F28,F29)</f>
+        <v>0.03</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <f aca="false">IF($D$4=1,G28,G29)</f>
+        <v>0.03</v>
+      </c>
+      <c r="H30" s="15" t="n">
+        <f aca="false">IF($D$4=1,H28,H29)</f>
+        <v>0.03</v>
+      </c>
+      <c r="I30" s="15" t="n">
+        <f aca="false">$H30</f>
+        <v>0.03</v>
+      </c>
+      <c r="J30" s="15" t="n">
+        <f aca="false">$H30</f>
+        <v>0.03</v>
+      </c>
+      <c r="K30" s="15" t="n">
+        <f aca="false">$H30</f>
+        <v>0.03</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <f aca="false">$H30</f>
+        <v>0.03</v>
+      </c>
+      <c r="M30" s="15" t="n">
+        <f aca="false">$H30</f>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="16" t="s">
+        <v>460</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E32" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="H32" s="10" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D33" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E33" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="G33" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="H33" s="10" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <f aca="false">IF($D$4=1,D32,D33)</f>
+        <v>35</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <f aca="false">IF($D$4=1,E32,E33)</f>
+        <v>30</v>
+      </c>
+      <c r="F34" s="11" t="n">
+        <f aca="false">IF($D$4=1,F32,F33)</f>
+        <v>30</v>
+      </c>
+      <c r="G34" s="11" t="n">
+        <f aca="false">IF($D$4=1,G32,G33)</f>
+        <v>30</v>
+      </c>
+      <c r="H34" s="11" t="n">
+        <f aca="false">IF($D$4=1,H32,H33)</f>
+        <v>30</v>
+      </c>
+      <c r="I34" s="11" t="n">
+        <f aca="false">$H34</f>
+        <v>30</v>
+      </c>
+      <c r="J34" s="11" t="n">
+        <f aca="false">$H34</f>
+        <v>30</v>
+      </c>
+      <c r="K34" s="11" t="n">
+        <f aca="false">$H34</f>
+        <v>30</v>
+      </c>
+      <c r="L34" s="11" t="n">
+        <f aca="false">$H34</f>
+        <v>30</v>
+      </c>
+      <c r="M34" s="11" t="n">
+        <f aca="false">$H34</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="16" t="s">
+        <v>462</v>
+      </c>
+      <c r="N35" s="6" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H36" s="13" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D37" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D38" s="15" t="n">
+        <f aca="false">IF($D$4=1,D36,D37)</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <f aca="false">IF($D$4=1,E36,E37)</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="15" t="n">
+        <f aca="false">IF($D$4=1,F36,F37)</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="15" t="n">
+        <f aca="false">IF($D$4=1,G36,G37)</f>
+        <v>0.05</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <f aca="false">IF($D$4=1,H36,H37)</f>
+        <v>0.05</v>
+      </c>
+      <c r="I38" s="15" t="n">
+        <f aca="false">$H38</f>
+        <v>0.05</v>
+      </c>
+      <c r="J38" s="15" t="n">
+        <f aca="false">$H38</f>
+        <v>0.05</v>
+      </c>
+      <c r="K38" s="15" t="n">
+        <f aca="false">$H38</f>
+        <v>0.05</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <f aca="false">$H38</f>
+        <v>0.05</v>
+      </c>
+      <c r="M38" s="15" t="n">
+        <f aca="false">$H38</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="16" t="s">
+        <v>464</v>
+      </c>
+      <c r="N39" s="6" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E40" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G40" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H40" s="13" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D41" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E41" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F41" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G41" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H41" s="13" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D42" s="15" t="n">
+        <f aca="false">IF($D$4=1,D40,D41)</f>
+        <v>0.03</v>
+      </c>
+      <c r="E42" s="15" t="n">
+        <f aca="false">IF($D$4=1,E40,E41)</f>
+        <v>0.03</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <f aca="false">IF($D$4=1,F40,F41)</f>
+        <v>0.03</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <f aca="false">IF($D$4=1,G40,G41)</f>
+        <v>0.03</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <f aca="false">IF($D$4=1,H40,H41)</f>
+        <v>0.03</v>
+      </c>
+      <c r="I42" s="15" t="n">
+        <f aca="false">$H42</f>
+        <v>0.03</v>
+      </c>
+      <c r="J42" s="15" t="n">
+        <f aca="false">$H42</f>
+        <v>0.03</v>
+      </c>
+      <c r="K42" s="15" t="n">
+        <f aca="false">$H42</f>
+        <v>0.03</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <f aca="false">$H42</f>
+        <v>0.03</v>
+      </c>
+      <c r="M42" s="15" t="n">
+        <f aca="false">$H42</f>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="16" t="s">
+        <v>466</v>
+      </c>
+      <c r="N43" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D44" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E44" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F44" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G44" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H44" s="13" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D45" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E45" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F45" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G45" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H45" s="13" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D46" s="15" t="n">
+        <f aca="false">IF($D$4=1,D44,D45)</f>
+        <v>0.75</v>
+      </c>
+      <c r="E46" s="15" t="n">
+        <f aca="false">IF($D$4=1,E44,E45)</f>
+        <v>0.75</v>
+      </c>
+      <c r="F46" s="15" t="n">
+        <f aca="false">IF($D$4=1,F44,F45)</f>
+        <v>0.75</v>
+      </c>
+      <c r="G46" s="15" t="n">
+        <f aca="false">IF($D$4=1,G44,G45)</f>
+        <v>0.75</v>
+      </c>
+      <c r="H46" s="15" t="n">
+        <f aca="false">IF($D$4=1,H44,H45)</f>
+        <v>0.75</v>
+      </c>
+      <c r="I46" s="15" t="n">
+        <f aca="false">$H46</f>
+        <v>0.75</v>
+      </c>
+      <c r="J46" s="15" t="n">
+        <f aca="false">$H46</f>
+        <v>0.75</v>
+      </c>
+      <c r="K46" s="15" t="n">
+        <f aca="false">$H46</f>
+        <v>0.75</v>
+      </c>
+      <c r="L46" s="15" t="n">
+        <f aca="false">$H46</f>
+        <v>0.75</v>
+      </c>
+      <c r="M46" s="15" t="n">
+        <f aca="false">$H46</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="16" t="s">
+        <v>468</v>
+      </c>
+      <c r="N47" s="6" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D48" s="13" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="E48" s="13" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="G48" s="13" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="H48" s="13" t="n">
+        <v>0.293</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D49" s="13" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="E49" s="13" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="F49" s="13" t="n">
+        <v>0.313</v>
+      </c>
+      <c r="G49" s="13" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="H49" s="13" t="n">
+        <v>0.333</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B50" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D50" s="15" t="n">
+        <f aca="false">IF($D$4=1,D48,D49)</f>
+        <v>0.293</v>
+      </c>
+      <c r="E50" s="15" t="n">
+        <f aca="false">IF($D$4=1,E48,E49)</f>
+        <v>0.293</v>
+      </c>
+      <c r="F50" s="15" t="n">
+        <f aca="false">IF($D$4=1,F48,F49)</f>
+        <v>0.293</v>
+      </c>
+      <c r="G50" s="15" t="n">
+        <f aca="false">IF($D$4=1,G48,G49)</f>
+        <v>0.293</v>
+      </c>
+      <c r="H50" s="15" t="n">
+        <f aca="false">IF($D$4=1,H48,H49)</f>
+        <v>0.293</v>
+      </c>
+      <c r="I50" s="15" t="n">
+        <f aca="false">$H50</f>
+        <v>0.293</v>
+      </c>
+      <c r="J50" s="15" t="n">
+        <f aca="false">$H50</f>
+        <v>0.293</v>
+      </c>
+      <c r="K50" s="15" t="n">
+        <f aca="false">$H50</f>
+        <v>0.293</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <f aca="false">$H50</f>
+        <v>0.293</v>
+      </c>
+      <c r="M50" s="15" t="n">
+        <f aca="false">$H50</f>
+        <v>0.293</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="16" t="s">
+        <v>470</v>
+      </c>
+      <c r="N51" s="6" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D52" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H52" s="13" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D53" s="13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E53" s="13" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F53" s="13" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G53" s="13" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H53" s="13" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D54" s="15" t="n">
+        <f aca="false">IF($D$4=1,D52,D53)</f>
+        <v>0.2</v>
+      </c>
+      <c r="E54" s="15" t="n">
+        <f aca="false">IF($D$4=1,E52,E53)</f>
+        <v>0.2</v>
+      </c>
+      <c r="F54" s="15" t="n">
+        <f aca="false">IF($D$4=1,F52,F53)</f>
+        <v>0.2</v>
+      </c>
+      <c r="G54" s="15" t="n">
+        <f aca="false">IF($D$4=1,G52,G53)</f>
+        <v>0.2</v>
+      </c>
+      <c r="H54" s="15" t="n">
+        <f aca="false">IF($D$4=1,H52,H53)</f>
+        <v>0.2</v>
+      </c>
+      <c r="I54" s="15" t="n">
+        <f aca="false">$H54</f>
+        <v>0.2</v>
+      </c>
+      <c r="J54" s="15" t="n">
+        <f aca="false">$H54</f>
+        <v>0.2</v>
+      </c>
+      <c r="K54" s="15" t="n">
+        <f aca="false">$H54</f>
+        <v>0.2</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <f aca="false">$H54</f>
+        <v>0.2</v>
+      </c>
+      <c r="M54" s="15" t="n">
+        <f aca="false">$H54</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="16" t="s">
+        <v>472</v>
+      </c>
+      <c r="N55" s="6" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D56" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E56" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G56" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H56" s="13" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D57" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E57" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F57" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G57" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H57" s="13" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D58" s="15" t="n">
+        <f aca="false">IF($D$4=1,D56,D57)</f>
+        <v>0.75</v>
+      </c>
+      <c r="E58" s="15" t="n">
+        <f aca="false">IF($D$4=1,E56,E57)</f>
+        <v>0.75</v>
+      </c>
+      <c r="F58" s="15" t="n">
+        <f aca="false">IF($D$4=1,F56,F57)</f>
+        <v>0.75</v>
+      </c>
+      <c r="G58" s="15" t="n">
+        <f aca="false">IF($D$4=1,G56,G57)</f>
+        <v>0.75</v>
+      </c>
+      <c r="H58" s="15" t="n">
+        <f aca="false">IF($D$4=1,H56,H57)</f>
+        <v>0.75</v>
+      </c>
+      <c r="I58" s="15" t="n">
+        <f aca="false">$H58</f>
+        <v>0.75</v>
+      </c>
+      <c r="J58" s="15" t="n">
+        <f aca="false">$H58</f>
+        <v>0.75</v>
+      </c>
+      <c r="K58" s="15" t="n">
+        <f aca="false">$H58</f>
+        <v>0.75</v>
+      </c>
+      <c r="L58" s="15" t="n">
+        <f aca="false">$H58</f>
+        <v>0.75</v>
+      </c>
+      <c r="M58" s="15" t="n">
+        <f aca="false">$H58</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="16" t="s">
+        <v>474</v>
+      </c>
+      <c r="N59" s="6" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D60" s="13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="E60" s="13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="G60" s="13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="H60" s="13" t="n">
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D61" s="13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="E61" s="13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="F61" s="13" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G61" s="13" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="H61" s="13" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="D62" s="15" t="n">
+        <f aca="false">IF($D$4=1,D60,D61)</f>
+        <v>0.065</v>
+      </c>
+      <c r="E62" s="15" t="n">
+        <f aca="false">IF($D$4=1,E60,E61)</f>
+        <v>0.065</v>
+      </c>
+      <c r="F62" s="15" t="n">
+        <f aca="false">IF($D$4=1,F60,F61)</f>
+        <v>0.065</v>
+      </c>
+      <c r="G62" s="15" t="n">
+        <f aca="false">IF($D$4=1,G60,G61)</f>
+        <v>0.065</v>
+      </c>
+      <c r="H62" s="15" t="n">
+        <f aca="false">IF($D$4=1,H60,H61)</f>
+        <v>0.065</v>
+      </c>
+      <c r="I62" s="15" t="n">
+        <f aca="false">$H62</f>
+        <v>0.065</v>
+      </c>
+      <c r="J62" s="15" t="n">
+        <f aca="false">$H62</f>
+        <v>0.065</v>
+      </c>
+      <c r="K62" s="15" t="n">
+        <f aca="false">$H62</f>
+        <v>0.065</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <f aca="false">$H62</f>
+        <v>0.065</v>
+      </c>
+      <c r="M62" s="15" t="n">
+        <f aca="false">$H62</f>
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="16" t="s">
+        <v>476</v>
+      </c>
+      <c r="N63" s="6" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="E64" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G64" s="13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H64" s="13" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="E65" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F65" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G65" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H65" s="13" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="E66" s="15" t="n">
+        <f aca="false">IF($D$4=1,E64,E65)</f>
+        <v>0.04</v>
+      </c>
+      <c r="F66" s="15" t="n">
+        <f aca="false">IF($D$4=1,F64,F65)</f>
+        <v>0.04</v>
+      </c>
+      <c r="G66" s="15" t="n">
+        <f aca="false">IF($D$4=1,G64,G65)</f>
+        <v>0.04</v>
+      </c>
+      <c r="H66" s="15" t="n">
+        <f aca="false">IF($D$4=1,H64,H65)</f>
+        <v>0.04</v>
+      </c>
+      <c r="I66" s="15" t="n">
+        <f aca="false">$H66</f>
+        <v>0.04</v>
+      </c>
+      <c r="J66" s="15" t="n">
+        <f aca="false">$H66</f>
+        <v>0.04</v>
+      </c>
+      <c r="K66" s="15" t="n">
+        <f aca="false">$H66</f>
+        <v>0.04</v>
+      </c>
+      <c r="L66" s="15" t="n">
+        <f aca="false">$H66</f>
+        <v>0.04</v>
+      </c>
+      <c r="M66" s="15" t="n">
+        <f aca="false">$H66</f>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="D68" s="5" t="n">
+        <f aca="false">DCF!C9</f>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="D69" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="N69" s="18" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="D70" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="N70" s="18" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B73" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="C73" s="10" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="D73" s="11" t="n">
+        <f aca="false">C73*(1+D14)</f>
+        <v>119.298</v>
+      </c>
+      <c r="E73" s="11" t="n">
+        <f aca="false">D73*(1+E14)</f>
+        <v>133.61376</v>
+      </c>
+      <c r="F73" s="11" t="n">
+        <f aca="false">E73*(1+F14)</f>
+        <v>148.3112736</v>
+      </c>
+      <c r="G73" s="11" t="n">
+        <f aca="false">F73*(1+G14)</f>
+        <v>163.14240096</v>
+      </c>
+      <c r="H73" s="11" t="n">
+        <f aca="false">G73*(1+H14)</f>
+        <v>177.8252170464</v>
+      </c>
+      <c r="I73" s="11" t="n">
+        <f aca="false">H73*(1+$H$14+($D$68-$H$14)*1/5)</f>
+        <v>191.695583976019</v>
+      </c>
+      <c r="J73" s="11" t="n">
+        <f aca="false">I73*(1+$H$14+($D$68-$H$14)*2/5)</f>
+        <v>204.347492518437</v>
+      </c>
+      <c r="K73" s="11" t="n">
+        <f aca="false">J73*(1+$H$14+($D$68-$H$14)*3/5)</f>
+        <v>215.382257114432</v>
+      </c>
+      <c r="L73" s="11" t="n">
+        <f aca="false">K73*(1+$H$14+($D$68-$H$14)*4/5)</f>
+        <v>224.428311913238</v>
+      </c>
+      <c r="M73" s="11" t="n">
+        <f aca="false">L73*(1+$H$14+($D$68-$H$14)*5/5)</f>
+        <v>231.161161270635</v>
+      </c>
+      <c r="N73" s="18" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="C74" s="11" t="n">
+        <f aca="false">C7*(1-0.03)-C73-C75</f>
+        <v>307.20689</v>
+      </c>
+      <c r="D74" s="11" t="n">
+        <f aca="false">D7*(1-D42)-D73-D75</f>
+        <v>373.34809</v>
+      </c>
+      <c r="E74" s="11" t="n">
+        <f aca="false">D74*(1+E18+E22+E26)*(1+E30)</f>
+        <v>415.312415316</v>
+      </c>
+      <c r="F74" s="11" t="n">
+        <f aca="false">E74*(1+F18+F22+F26)*(1+F30)</f>
+        <v>461.993530797518</v>
+      </c>
+      <c r="G74" s="11" t="n">
+        <f aca="false">F74*(1+G18+G22+G26)*(1+G30)</f>
+        <v>513.92160365916</v>
+      </c>
+      <c r="H74" s="11" t="n">
+        <f aca="false">G74*(1+H18+H22+H26)*(1+H30)</f>
+        <v>571.686391910449</v>
+      </c>
+      <c r="I74" s="11" t="n">
+        <f aca="false">H74*(1+($H$74/$G$74-1)+($D$68-($H$74/$G$74-1))*1/5)</f>
+        <v>626.5225506225</v>
+      </c>
+      <c r="J74" s="11" t="n">
+        <f aca="false">I74*(1+($H$74/$G$74-1)+($D$68-($H$74/$G$74-1))*2/5)</f>
+        <v>676.293502043951</v>
+      </c>
+      <c r="K74" s="11" t="n">
+        <f aca="false">J74*(1+($H$74/$G$74-1)+($D$68-($H$74/$G$74-1))*3/5)</f>
+        <v>718.872940932638</v>
+      </c>
+      <c r="L74" s="11" t="n">
+        <f aca="false">K74*(1+($H$74/$G$74-1)+($D$68-($H$74/$G$74-1))*4/5)</f>
+        <v>752.286155227187</v>
+      </c>
+      <c r="M74" s="11" t="n">
+        <f aca="false">L74*(1+($H$74/$G$74-1)+($D$68-($H$74/$G$74-1))*5/5)</f>
+        <v>774.854739884003</v>
+      </c>
+      <c r="N74" s="6" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C75" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="D75" s="11" t="n">
+        <f aca="false">D87+0.5*D88</f>
+        <v>42.5</v>
+      </c>
+      <c r="E75" s="11" t="n">
+        <f aca="false">E87+0.5*E88</f>
+        <v>76.8</v>
+      </c>
+      <c r="F75" s="11" t="n">
+        <f aca="false">F87+0.5*F88</f>
+        <v>109.554</v>
+      </c>
+      <c r="G75" s="11" t="n">
+        <f aca="false">G87+0.5*G88</f>
+        <v>136.876089</v>
+      </c>
+      <c r="H75" s="11" t="n">
+        <f aca="false">H87+0.5*H88</f>
+        <v>163.6107530865</v>
+      </c>
+      <c r="I75" s="11" t="n">
+        <f aca="false">H75*(1+($H$75/$G$75-1)+($D$68-($H$75/$G$75-1))*1/5)</f>
+        <v>190.157604668228</v>
+      </c>
+      <c r="J75" s="11" t="n">
+        <f aca="false">I75*(1+($H$75/$G$75-1)+($D$68-($H$75/$G$75-1))*2/5)</f>
+        <v>214.724467922381</v>
+      </c>
+      <c r="K75" s="11" t="n">
+        <f aca="false">J75*(1+($H$75/$G$75-1)+($D$68-($H$75/$G$75-1))*3/5)</f>
+        <v>235.365518130177</v>
+      </c>
+      <c r="L75" s="11" t="n">
+        <f aca="false">K75*(1+($H$75/$G$75-1)+($D$68-($H$75/$G$75-1))*4/5)</f>
+        <v>250.208618238932</v>
+      </c>
+      <c r="M75" s="11" t="n">
+        <f aca="false">L75*(1+($H$75/$G$75-1)+($D$68-($H$75/$G$75-1))*5/5)</f>
+        <v>257.7148767861</v>
+      </c>
+      <c r="N75" s="6" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="16" t="s">
+        <v>489</v>
+      </c>
+      <c r="C76" s="11" t="n">
+        <f aca="false">C73+C74+C75</f>
+        <v>421.30689</v>
+      </c>
+      <c r="D76" s="11" t="n">
+        <f aca="false">D73+D74+D75</f>
+        <v>535.14609</v>
+      </c>
+      <c r="E76" s="11" t="n">
+        <f aca="false">E73+E74+E75</f>
+        <v>625.726175316</v>
+      </c>
+      <c r="F76" s="11" t="n">
+        <f aca="false">F73+F74+F75</f>
+        <v>719.858804397518</v>
+      </c>
+      <c r="G76" s="11" t="n">
+        <f aca="false">G73+G74+G75</f>
+        <v>813.94009361916</v>
+      </c>
+      <c r="H76" s="11" t="n">
+        <f aca="false">H73+H74+H75</f>
+        <v>913.122362043349</v>
+      </c>
+      <c r="I76" s="11" t="n">
+        <f aca="false">I73+I74+I75</f>
+        <v>1008.37573926675</v>
+      </c>
+      <c r="J76" s="11" t="n">
+        <f aca="false">J73+J74+J75</f>
+        <v>1095.36546248477</v>
+      </c>
+      <c r="K76" s="11" t="n">
+        <f aca="false">K73+K74+K75</f>
+        <v>1169.62071617725</v>
+      </c>
+      <c r="L76" s="11" t="n">
+        <f aca="false">L73+L74+L75</f>
+        <v>1226.92308537936</v>
+      </c>
+      <c r="M76" s="11" t="n">
+        <f aca="false">M73+M74+M75</f>
+        <v>1263.73077794074</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="C77" s="11" t="n">
+        <f aca="false">C7*0.03</f>
+        <v>13.03011</v>
+      </c>
+      <c r="D77" s="11" t="n">
+        <f aca="false">D7*D42</f>
+        <v>16.55091</v>
+      </c>
+      <c r="E77" s="11" t="n">
+        <f aca="false">E76*E42/(1-E42)</f>
+        <v>19.3523559376082</v>
+      </c>
+      <c r="F77" s="11" t="n">
+        <f aca="false">F76*F42/(1-F42)</f>
+        <v>22.2636743628098</v>
+      </c>
+      <c r="G77" s="11" t="n">
+        <f aca="false">G76*G42/(1-G42)</f>
+        <v>25.1734049572936</v>
+      </c>
+      <c r="H77" s="11" t="n">
+        <f aca="false">H76*H42/(1-H42)</f>
+        <v>28.2408977951551</v>
+      </c>
+      <c r="I77" s="11" t="n">
+        <f aca="false">I76*I42/(1-I42)</f>
+        <v>31.1868785340231</v>
+      </c>
+      <c r="J77" s="11" t="n">
+        <f aca="false">J76*J42/(1-J42)</f>
+        <v>33.8772823448898</v>
+      </c>
+      <c r="K77" s="11" t="n">
+        <f aca="false">K76*K42/(1-K42)</f>
+        <v>36.1738365828015</v>
+      </c>
+      <c r="L77" s="11" t="n">
+        <f aca="false">L76*L42/(1-L42)</f>
+        <v>37.9460748055471</v>
+      </c>
+      <c r="M77" s="11" t="n">
+        <f aca="false">M76*M42/(1-M42)</f>
+        <v>39.0844570497136</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B78" s="16" t="s">
+        <v>491</v>
+      </c>
+      <c r="C78" s="12" t="n">
+        <f aca="false">C7</f>
+        <v>434.337</v>
+      </c>
+      <c r="D78" s="12" t="n">
+        <f aca="false">D7</f>
+        <v>551.697</v>
+      </c>
+      <c r="E78" s="11" t="n">
+        <f aca="false">E76+E77</f>
+        <v>645.078531253608</v>
+      </c>
+      <c r="F78" s="11" t="n">
+        <f aca="false">F76+F77</f>
+        <v>742.122478760328</v>
+      </c>
+      <c r="G78" s="11" t="n">
+        <f aca="false">G76+G77</f>
+        <v>839.113498576453</v>
+      </c>
+      <c r="H78" s="11" t="n">
+        <f aca="false">H76+H77</f>
+        <v>941.363259838504</v>
+      </c>
+      <c r="I78" s="11" t="n">
+        <f aca="false">I76+I77</f>
+        <v>1039.56261780077</v>
+      </c>
+      <c r="J78" s="11" t="n">
+        <f aca="false">J76+J77</f>
+        <v>1129.24274482966</v>
+      </c>
+      <c r="K78" s="11" t="n">
+        <f aca="false">K76+K77</f>
+        <v>1205.79455276005</v>
+      </c>
+      <c r="L78" s="11" t="n">
+        <f aca="false">L76+L77</f>
+        <v>1264.8691601849</v>
+      </c>
+      <c r="M78" s="11" t="n">
+        <f aca="false">M76+M77</f>
+        <v>1302.81523499045</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="D79" s="15" t="n">
+        <f aca="false">D78/C78-1</f>
+        <v>0.270204933035868</v>
+      </c>
+      <c r="E79" s="15" t="n">
+        <f aca="false">E78/D78-1</f>
+        <v>0.169262350989054</v>
+      </c>
+      <c r="F79" s="15" t="n">
+        <f aca="false">F78/E78-1</f>
+        <v>0.1504374162292</v>
+      </c>
+      <c r="G79" s="15" t="n">
+        <f aca="false">G78/F78-1</f>
+        <v>0.130694087016664</v>
+      </c>
+      <c r="H79" s="15" t="n">
+        <f aca="false">H78/G78-1</f>
+        <v>0.121854506494672</v>
+      </c>
+      <c r="I79" s="15" t="n">
+        <f aca="false">I78/H78-1</f>
+        <v>0.104316114885461</v>
+      </c>
+      <c r="J79" s="15" t="n">
+        <f aca="false">J78/I78-1</f>
+        <v>0.0862671718790828</v>
+      </c>
+      <c r="K79" s="15" t="n">
+        <f aca="false">K78/J78-1</f>
+        <v>0.0677903916415577</v>
+      </c>
+      <c r="L79" s="15" t="n">
+        <f aca="false">L78/K78-1</f>
+        <v>0.0489922659624187</v>
+      </c>
+      <c r="M79" s="15" t="n">
+        <f aca="false">M78/L78-1</f>
+        <v>0.0300000000000003</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="D80" s="24" t="n">
+        <f aca="false">D78/D7-1</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="24" t="n">
+        <f aca="false">E78/E7-1</f>
+        <v>-0.0440136885707473</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="C81" s="15" t="n">
+        <f aca="false">(C74+C75)/C78</f>
+        <v>0.737231435498242</v>
+      </c>
+      <c r="D81" s="15" t="n">
+        <f aca="false">(D74+D75)/D78</f>
+        <v>0.753761738780526</v>
+      </c>
+      <c r="E81" s="15" t="n">
+        <f aca="false">(E74+E75)/E78</f>
+        <v>0.76287210234645</v>
+      </c>
+      <c r="F81" s="15" t="n">
+        <f aca="false">(F74+F75)/F78</f>
+        <v>0.770152565318133</v>
+      </c>
+      <c r="G81" s="15" t="n">
+        <f aca="false">(G74+G75)/G78</f>
+        <v>0.77557767067653</v>
+      </c>
+      <c r="H81" s="15" t="n">
+        <f aca="false">(H74+H75)/H78</f>
+        <v>0.781098197015989</v>
+      </c>
+      <c r="I81" s="15" t="n">
+        <f aca="false">(I74+I75)/I78</f>
+        <v>0.785599771775598</v>
+      </c>
+      <c r="J81" s="15" t="n">
+        <f aca="false">(J74+J75)/J78</f>
+        <v>0.789040243159356</v>
+      </c>
+      <c r="K81" s="15" t="n">
+        <f aca="false">(K74+K75)/K78</f>
+        <v>0.79137731786777</v>
+      </c>
+      <c r="L81" s="15" t="n">
+        <f aca="false">(L74+L75)/L78</f>
+        <v>0.792567962776142</v>
+      </c>
+      <c r="M81" s="15" t="n">
+        <f aca="false">(M74+M75)/M78</f>
+        <v>0.792567962776142</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="C82" s="12" t="n">
+        <f aca="false">$D$70</f>
+        <v>60</v>
+      </c>
+      <c r="D82" s="11" t="n">
+        <f aca="false">C82*(1+IF(D30="",0.03,D30))</f>
+        <v>61.8</v>
+      </c>
+      <c r="E82" s="11" t="n">
+        <f aca="false">D82*(1+IF(E30="",0.03,E30))</f>
+        <v>63.654</v>
+      </c>
+      <c r="F82" s="11" t="n">
+        <f aca="false">E82*(1+IF(F30="",0.03,F30))</f>
+        <v>65.56362</v>
+      </c>
+      <c r="G82" s="11" t="n">
+        <f aca="false">F82*(1+IF(G30="",0.03,G30))</f>
+        <v>67.5305286</v>
+      </c>
+      <c r="H82" s="11" t="n">
+        <f aca="false">G82*(1+IF(H30="",0.03,H30))</f>
+        <v>69.556444458</v>
+      </c>
+      <c r="I82" s="11" t="n">
+        <f aca="false">H82*1.03</f>
+        <v>71.64313779174</v>
+      </c>
+      <c r="J82" s="11" t="n">
+        <f aca="false">I82*1.03</f>
+        <v>73.7924319254922</v>
+      </c>
+      <c r="K82" s="11" t="n">
+        <f aca="false">J82*1.03</f>
+        <v>76.006204883257</v>
+      </c>
+      <c r="L82" s="11" t="n">
+        <f aca="false">K82*1.03</f>
+        <v>78.2863910297547</v>
+      </c>
+      <c r="M82" s="11" t="n">
+        <f aca="false">L82*1.03</f>
+        <v>80.6349827606473</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="C83" s="33" t="n">
+        <f aca="false">C74/C82</f>
+        <v>5.12011483333333</v>
+      </c>
+      <c r="D83" s="33" t="n">
+        <f aca="false">D74/D82</f>
+        <v>6.04123122977346</v>
+      </c>
+      <c r="E83" s="33" t="n">
+        <f aca="false">E74/E82</f>
+        <v>6.52452972815534</v>
+      </c>
+      <c r="F83" s="33" t="n">
+        <f aca="false">F74/F82</f>
+        <v>7.04649210640777</v>
+      </c>
+      <c r="G83" s="33" t="n">
+        <f aca="false">G74/G82</f>
+        <v>7.61021147492039</v>
+      </c>
+      <c r="H83" s="33" t="n">
+        <f aca="false">H74/H82</f>
+        <v>8.21902839291402</v>
+      </c>
+      <c r="I83" s="33" t="n">
+        <f aca="false">I74/I82</f>
+        <v>8.74504621006052</v>
+      </c>
+      <c r="J83" s="33" t="n">
+        <f aca="false">J74/J82</f>
+        <v>9.16480842814342</v>
+      </c>
+      <c r="K83" s="33" t="n">
+        <f aca="false">K74/K82</f>
+        <v>9.45808229784401</v>
+      </c>
+      <c r="L83" s="33" t="n">
+        <f aca="false">L74/L82</f>
+        <v>9.60941161460952</v>
+      </c>
+      <c r="M83" s="33" t="n">
+        <f aca="false">M74/M82</f>
+        <v>9.60941161460952</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B85" s="16" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B86" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="D86" s="12" t="n">
+        <f aca="false">$D$69</f>
+        <v>25</v>
+      </c>
+      <c r="E86" s="11" t="n">
+        <f aca="false">D89</f>
+        <v>60</v>
+      </c>
+      <c r="F86" s="11" t="n">
+        <f aca="false">E89</f>
+        <v>91.8</v>
+      </c>
+      <c r="G86" s="11" t="n">
+        <f aca="false">F89</f>
+        <v>124.554</v>
+      </c>
+      <c r="H86" s="11" t="n">
+        <f aca="false">G89</f>
+        <v>151.876089</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B87" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="D87" s="11" t="n">
+        <f aca="false">D86</f>
+        <v>25</v>
+      </c>
+      <c r="E87" s="11" t="n">
+        <f aca="false">E86*(1+E30)*(1-E38)</f>
+        <v>61.8</v>
+      </c>
+      <c r="F87" s="11" t="n">
+        <f aca="false">F86*(1+F30)*(1-F38)</f>
+        <v>94.554</v>
+      </c>
+      <c r="G87" s="11" t="n">
+        <f aca="false">G86*(1+G30)*(1-G38)</f>
+        <v>121.876089</v>
+      </c>
+      <c r="H87" s="11" t="n">
+        <f aca="false">H86*(1+H30)*(1-H38)</f>
+        <v>148.6107530865</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B88" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="D88" s="11" t="n">
+        <f aca="false">D34</f>
+        <v>35</v>
+      </c>
+      <c r="E88" s="11" t="n">
+        <f aca="false">E34</f>
+        <v>30</v>
+      </c>
+      <c r="F88" s="11" t="n">
+        <f aca="false">F34</f>
+        <v>30</v>
+      </c>
+      <c r="G88" s="11" t="n">
+        <f aca="false">G34</f>
+        <v>30</v>
+      </c>
+      <c r="H88" s="11" t="n">
+        <f aca="false">H34</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B89" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="D89" s="11" t="n">
+        <f aca="false">D87+D88</f>
+        <v>60</v>
+      </c>
+      <c r="E89" s="11" t="n">
+        <f aca="false">E87+E88</f>
+        <v>91.8</v>
+      </c>
+      <c r="F89" s="11" t="n">
+        <f aca="false">F87+F88</f>
+        <v>124.554</v>
+      </c>
+      <c r="G89" s="11" t="n">
+        <f aca="false">G87+G88</f>
+        <v>151.876089</v>
+      </c>
+      <c r="H89" s="11" t="n">
+        <f aca="false">H87+H88</f>
+        <v>178.6107530865</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B91" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B92" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="D92" s="11" t="n">
+        <f aca="false">D73*D46</f>
+        <v>89.4735</v>
+      </c>
+      <c r="E92" s="11" t="n">
+        <f aca="false">E73*E46</f>
+        <v>100.21032</v>
+      </c>
+      <c r="F92" s="11" t="n">
+        <f aca="false">F73*F46</f>
+        <v>111.2334552</v>
+      </c>
+      <c r="G92" s="11" t="n">
+        <f aca="false">G73*G46</f>
+        <v>122.35680072</v>
+      </c>
+      <c r="H92" s="11" t="n">
+        <f aca="false">H73*H46</f>
+        <v>133.3689127848</v>
+      </c>
+      <c r="I92" s="11" t="n">
+        <f aca="false">I73*I46</f>
+        <v>143.771687982014</v>
+      </c>
+      <c r="J92" s="11" t="n">
+        <f aca="false">J73*J46</f>
+        <v>153.260619388827</v>
+      </c>
+      <c r="K92" s="11" t="n">
+        <f aca="false">K73*K46</f>
+        <v>161.536692835824</v>
+      </c>
+      <c r="L92" s="11" t="n">
+        <f aca="false">L73*L46</f>
+        <v>168.321233934929</v>
+      </c>
+      <c r="M92" s="11" t="n">
+        <f aca="false">M73*M46</f>
+        <v>173.370870952977</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B93" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="D93" s="11" t="n">
+        <f aca="false">D74*D50</f>
+        <v>109.39099037</v>
+      </c>
+      <c r="E93" s="11" t="n">
+        <f aca="false">E74*E50</f>
+        <v>121.686537687588</v>
+      </c>
+      <c r="F93" s="11" t="n">
+        <f aca="false">F74*F50</f>
+        <v>135.364104523673</v>
+      </c>
+      <c r="G93" s="11" t="n">
+        <f aca="false">G74*G50</f>
+        <v>150.579029872134</v>
+      </c>
+      <c r="H93" s="11" t="n">
+        <f aca="false">H74*H50</f>
+        <v>167.504112829762</v>
+      </c>
+      <c r="I93" s="11" t="n">
+        <f aca="false">I74*I50</f>
+        <v>183.571107332392</v>
+      </c>
+      <c r="J93" s="11" t="n">
+        <f aca="false">J74*J50</f>
+        <v>198.153996098878</v>
+      </c>
+      <c r="K93" s="11" t="n">
+        <f aca="false">K74*K50</f>
+        <v>210.629771693263</v>
+      </c>
+      <c r="L93" s="11" t="n">
+        <f aca="false">L74*L50</f>
+        <v>220.419843481566</v>
+      </c>
+      <c r="M93" s="11" t="n">
+        <f aca="false">M74*M50</f>
+        <v>227.032438786013</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B94" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="D94" s="11" t="n">
+        <f aca="false">D75*D54</f>
+        <v>8.5</v>
+      </c>
+      <c r="E94" s="11" t="n">
+        <f aca="false">E75*E54</f>
+        <v>15.36</v>
+      </c>
+      <c r="F94" s="11" t="n">
+        <f aca="false">F75*F54</f>
+        <v>21.9108</v>
+      </c>
+      <c r="G94" s="11" t="n">
+        <f aca="false">G75*G54</f>
+        <v>27.3752178</v>
+      </c>
+      <c r="H94" s="11" t="n">
+        <f aca="false">H75*H54</f>
+        <v>32.7221506173</v>
+      </c>
+      <c r="I94" s="11" t="n">
+        <f aca="false">I75*I54</f>
+        <v>38.0315209336457</v>
+      </c>
+      <c r="J94" s="11" t="n">
+        <f aca="false">J75*J54</f>
+        <v>42.9448935844763</v>
+      </c>
+      <c r="K94" s="11" t="n">
+        <f aca="false">K75*K54</f>
+        <v>47.0731036260354</v>
+      </c>
+      <c r="L94" s="11" t="n">
+        <f aca="false">L75*L54</f>
+        <v>50.0417236477864</v>
+      </c>
+      <c r="M94" s="11" t="n">
+        <f aca="false">M75*M54</f>
+        <v>51.54297535722</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B95" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="D95" s="11" t="n">
+        <f aca="false">D77*D58</f>
+        <v>12.4131825</v>
+      </c>
+      <c r="E95" s="11" t="n">
+        <f aca="false">E77*E58</f>
+        <v>14.5142669532062</v>
+      </c>
+      <c r="F95" s="11" t="n">
+        <f aca="false">F77*F58</f>
+        <v>16.6977557721074</v>
+      </c>
+      <c r="G95" s="11" t="n">
+        <f aca="false">G77*G58</f>
+        <v>18.8800537179702</v>
+      </c>
+      <c r="H95" s="11" t="n">
+        <f aca="false">H77*H58</f>
+        <v>21.1806733463663</v>
+      </c>
+      <c r="I95" s="11" t="n">
+        <f aca="false">I77*I58</f>
+        <v>23.3901589005173</v>
+      </c>
+      <c r="J95" s="11" t="n">
+        <f aca="false">J77*J58</f>
+        <v>25.4079617586673</v>
+      </c>
+      <c r="K95" s="11" t="n">
+        <f aca="false">K77*K58</f>
+        <v>27.1303774371011</v>
+      </c>
+      <c r="L95" s="11" t="n">
+        <f aca="false">L77*L58</f>
+        <v>28.4595561041604</v>
+      </c>
+      <c r="M95" s="11" t="n">
+        <f aca="false">M77*M58</f>
+        <v>29.3133427872852</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B96" s="16" t="s">
+        <v>506</v>
+      </c>
+      <c r="D96" s="11" t="n">
+        <f aca="false">SUM(D92:D95)</f>
+        <v>219.77767287</v>
+      </c>
+      <c r="E96" s="11" t="n">
+        <f aca="false">SUM(E92:E95)</f>
+        <v>251.771124640794</v>
+      </c>
+      <c r="F96" s="11" t="n">
+        <f aca="false">SUM(F92:F95)</f>
+        <v>285.20611549578</v>
+      </c>
+      <c r="G96" s="11" t="n">
+        <f aca="false">SUM(G92:G95)</f>
+        <v>319.191102110104</v>
+      </c>
+      <c r="H96" s="11" t="n">
+        <f aca="false">SUM(H92:H95)</f>
+        <v>354.775849578228</v>
+      </c>
+      <c r="I96" s="11" t="n">
+        <f aca="false">SUM(I92:I95)</f>
+        <v>388.76447514857</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <f aca="false">SUM(J92:J95)</f>
+        <v>419.767470830849</v>
+      </c>
+      <c r="K96" s="11" t="n">
+        <f aca="false">SUM(K92:K95)</f>
+        <v>446.369945592224</v>
+      </c>
+      <c r="L96" s="11" t="n">
+        <f aca="false">SUM(L92:L95)</f>
+        <v>467.242357168441</v>
+      </c>
+      <c r="M96" s="11" t="n">
+        <f aca="false">SUM(M92:M95)</f>
+        <v>481.259627883495</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B97" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="D97" s="15" t="n">
+        <f aca="false">D96/D78</f>
+        <v>0.398366626735328</v>
+      </c>
+      <c r="E97" s="15" t="n">
+        <f aca="false">E96/E78</f>
+        <v>0.390295308931638</v>
+      </c>
+      <c r="F97" s="15" t="n">
+        <f aca="false">F96/F78</f>
+        <v>0.384311382094503</v>
+      </c>
+      <c r="G97" s="15" t="n">
+        <f aca="false">G96/G78</f>
+        <v>0.380390856125671</v>
+      </c>
+      <c r="H97" s="15" t="n">
+        <f aca="false">H96/H78</f>
+        <v>0.376874544306192</v>
+      </c>
+      <c r="I97" s="15" t="n">
+        <f aca="false">I96/I78</f>
+        <v>0.373969271779909</v>
+      </c>
+      <c r="J97" s="15" t="n">
+        <f aca="false">J96/J78</f>
+        <v>0.371724744527067</v>
+      </c>
+      <c r="K97" s="15" t="n">
+        <f aca="false">K96/K78</f>
+        <v>0.370187395995851</v>
+      </c>
+      <c r="L97" s="15" t="n">
+        <f aca="false">L96/L78</f>
+        <v>0.369399754437951</v>
+      </c>
+      <c r="M97" s="15" t="n">
+        <f aca="false">M96/M78</f>
+        <v>0.369399754437951</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B98" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="D98" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E98" s="13" t="n">
+        <v>0.408</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B100" s="3" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B101" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="D101" s="11" t="n">
+        <f aca="false">D62*(D74+D75)</f>
+        <v>27.03012585</v>
+      </c>
+      <c r="E101" s="11" t="n">
+        <f aca="false">E62*(E74+E75)</f>
+        <v>31.98730699554</v>
+      </c>
+      <c r="F101" s="11" t="n">
+        <f aca="false">F62*(F74+F75)</f>
+        <v>37.1505895018387</v>
+      </c>
+      <c r="G101" s="11" t="n">
+        <f aca="false">G62*(G74+G75)</f>
+        <v>42.3018500228454</v>
+      </c>
+      <c r="H101" s="11" t="n">
+        <f aca="false">H62*(H74+H75)</f>
+        <v>47.7943144248017</v>
+      </c>
+      <c r="I101" s="11" t="n">
+        <f aca="false">I62*(I74+I75)</f>
+        <v>53.0842100938973</v>
+      </c>
+      <c r="J101" s="11" t="n">
+        <f aca="false">J62*(J74+J75)</f>
+        <v>57.9161680478116</v>
+      </c>
+      <c r="K101" s="11" t="n">
+        <f aca="false">K62*(K74+K75)</f>
+        <v>62.025499839083</v>
+      </c>
+      <c r="L101" s="11" t="n">
+        <f aca="false">L62*(L74+L75)</f>
+        <v>65.1621602752978</v>
+      </c>
+      <c r="M101" s="11" t="n">
+        <f aca="false">M62*(M74+M75)</f>
+        <v>67.1170250835567</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B102" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="D102" s="11" t="n">
+        <f aca="false">(D96-D8)-D101</f>
+        <v>200.18254702</v>
+      </c>
+      <c r="E102" s="11" t="n">
+        <f aca="false">D102*(1+E66)</f>
+        <v>208.1898489008</v>
+      </c>
+      <c r="F102" s="11" t="n">
+        <f aca="false">E102*(1+F66)</f>
+        <v>216.517442856832</v>
+      </c>
+      <c r="G102" s="11" t="n">
+        <f aca="false">F102*(1+G66)</f>
+        <v>225.178140571105</v>
+      </c>
+      <c r="H102" s="11" t="n">
+        <f aca="false">G102*(1+H66)</f>
+        <v>234.18526619395</v>
+      </c>
+      <c r="I102" s="11" t="n">
+        <f aca="false">H102*(1+I66)</f>
+        <v>243.552676841708</v>
+      </c>
+      <c r="J102" s="11" t="n">
+        <f aca="false">I102*(1+J66)</f>
+        <v>253.294783915376</v>
+      </c>
+      <c r="K102" s="11" t="n">
+        <f aca="false">J102*(1+K66)</f>
+        <v>263.426575271991</v>
+      </c>
+      <c r="L102" s="11" t="n">
+        <f aca="false">K102*(1+L66)</f>
+        <v>273.963638282871</v>
+      </c>
+      <c r="M102" s="11" t="n">
+        <f aca="false">L102*(1+M66)</f>
+        <v>284.922183814185</v>
+      </c>
+      <c r="N102" s="6" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B103" s="16" t="s">
+        <v>513</v>
+      </c>
+      <c r="D103" s="11" t="n">
+        <f aca="false">D101+D102</f>
+        <v>227.21267287</v>
+      </c>
+      <c r="E103" s="11" t="n">
+        <f aca="false">E101+E102</f>
+        <v>240.17715589634</v>
+      </c>
+      <c r="F103" s="11" t="n">
+        <f aca="false">F101+F102</f>
+        <v>253.668032358671</v>
+      </c>
+      <c r="G103" s="11" t="n">
+        <f aca="false">G101+G102</f>
+        <v>267.479990593951</v>
+      </c>
+      <c r="H103" s="11" t="n">
+        <f aca="false">H101+H102</f>
+        <v>281.979580618751</v>
+      </c>
+      <c r="I103" s="11" t="n">
+        <f aca="false">I101+I102</f>
+        <v>296.636886935605</v>
+      </c>
+      <c r="J103" s="11" t="n">
+        <f aca="false">J101+J102</f>
+        <v>311.210951963187</v>
+      </c>
+      <c r="K103" s="11" t="n">
+        <f aca="false">K101+K102</f>
+        <v>325.452075111074</v>
+      </c>
+      <c r="L103" s="11" t="n">
+        <f aca="false">L101+L102</f>
+        <v>339.125798558168</v>
+      </c>
+      <c r="M103" s="11" t="n">
+        <f aca="false">M101+M102</f>
+        <v>352.039208897742</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B104" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="D104" s="15" t="n">
+        <f aca="false">D103/D78</f>
+        <v>0.411843227115609</v>
+      </c>
+      <c r="E104" s="15" t="n">
+        <f aca="false">E103/E78</f>
+        <v>0.372322351868684</v>
+      </c>
+      <c r="F104" s="15" t="n">
+        <f aca="false">F103/F78</f>
+        <v>0.341814241744042</v>
+      </c>
+      <c r="G104" s="15" t="n">
+        <f aca="false">G103/G78</f>
+        <v>0.318764971660839</v>
+      </c>
+      <c r="H104" s="15" t="n">
+        <f aca="false">H103/H78</f>
+        <v>0.299543855861898</v>
+      </c>
+      <c r="I104" s="15" t="n">
+        <f aca="false">I103/I78</f>
+        <v>0.285347781707609</v>
+      </c>
+      <c r="J104" s="15" t="n">
+        <f aca="false">J103/J78</f>
+        <v>0.275592606982064</v>
+      </c>
+      <c r="K104" s="15" t="n">
+        <f aca="false">K103/K78</f>
+        <v>0.269906738561821</v>
+      </c>
+      <c r="L104" s="15" t="n">
+        <f aca="false">L103/L78</f>
+        <v>0.268111366165804</v>
+      </c>
+      <c r="M104" s="15" t="n">
+        <f aca="false">M103/M78</f>
+        <v>0.270214224889934</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B105" s="16" t="s">
+        <v>515</v>
+      </c>
+      <c r="D105" s="11" t="n">
+        <f aca="false">D96-D103</f>
+        <v>-7.435</v>
+      </c>
+      <c r="E105" s="11" t="n">
+        <f aca="false">E96-E103</f>
+        <v>11.5939687444542</v>
+      </c>
+      <c r="F105" s="11" t="n">
+        <f aca="false">F96-F103</f>
+        <v>31.5380831371095</v>
+      </c>
+      <c r="G105" s="11" t="n">
+        <f aca="false">G96-G103</f>
+        <v>51.7111115161533</v>
+      </c>
+      <c r="H105" s="11" t="n">
+        <f aca="false">H96-H103</f>
+        <v>72.7962689594767</v>
+      </c>
+      <c r="I105" s="11" t="n">
+        <f aca="false">I96-I103</f>
+        <v>92.127588212965</v>
+      </c>
+      <c r="J105" s="11" t="n">
+        <f aca="false">J96-J103</f>
+        <v>108.556518867661</v>
+      </c>
+      <c r="K105" s="11" t="n">
+        <f aca="false">K96-K103</f>
+        <v>120.91787048115</v>
+      </c>
+      <c r="L105" s="11" t="n">
+        <f aca="false">L96-L103</f>
+        <v>128.116558610273</v>
+      </c>
+      <c r="M105" s="11" t="n">
+        <f aca="false">M96-M103</f>
+        <v>129.220418985752</v>
+      </c>
+      <c r="N105" s="6" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B106" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="D106" s="15" t="n">
+        <f aca="false">D105/D78</f>
+        <v>-0.0134766003802812</v>
+      </c>
+      <c r="E106" s="15" t="n">
+        <f aca="false">E105/E78</f>
+        <v>0.0179729570629534</v>
+      </c>
+      <c r="F106" s="15" t="n">
+        <f aca="false">F105/F78</f>
+        <v>0.0424971403504608</v>
+      </c>
+      <c r="G106" s="15" t="n">
+        <f aca="false">G105/G78</f>
+        <v>0.0616258844648318</v>
+      </c>
+      <c r="H106" s="15" t="n">
+        <f aca="false">H105/H78</f>
+        <v>0.0773306884442944</v>
+      </c>
+      <c r="I106" s="15" t="n">
+        <f aca="false">I105/I78</f>
+        <v>0.0886214900722998</v>
+      </c>
+      <c r="J106" s="15" t="n">
+        <f aca="false">J105/J78</f>
+        <v>0.0961321375450027</v>
+      </c>
+      <c r="K106" s="15" t="n">
+        <f aca="false">K105/K78</f>
+        <v>0.10028065743403</v>
+      </c>
+      <c r="L106" s="15" t="n">
+        <f aca="false">L105/L78</f>
+        <v>0.101288388272147</v>
+      </c>
+      <c r="M106" s="15" t="n">
+        <f aca="false">M105/M78</f>
+        <v>0.0991855295480172</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B107" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D107" s="11" t="n">
+        <f aca="false">D105-D8</f>
+        <v>0</v>
+      </c>
+      <c r="E107" s="11" t="n">
+        <f aca="false">E105-E8</f>
+        <v>-17.8490312555458</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:N2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M59"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="1" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="C5" s="32" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="D6" s="18"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <f aca="false">C4+C5*C6</f>
+        <v>0.114</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <f aca="false">C7</f>
+        <v>0.114</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D9" s="18"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D10" s="18"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>2030</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="C12" s="13" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="C15" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>336</v>
+      </c>
+      <c r="D16" s="18"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="C17" s="37" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="4" t="s">
+        <v>545</v>
+      </c>
+      <c r="C18" s="38" t="n">
+        <f aca="false">Consensus_Check!C29</f>
+        <v>28.37</v>
+      </c>
+      <c r="D18" s="18"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="C19" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="M21" s="9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="12" t="n">
+        <f aca="false">Revenue_Build!D78</f>
+        <v>551.697</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <f aca="false">Revenue_Build!E78</f>
+        <v>645.078531253608</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <f aca="false">Revenue_Build!F78</f>
+        <v>742.122478760328</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <f aca="false">Revenue_Build!G78</f>
+        <v>839.113498576453</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <f aca="false">Revenue_Build!H78</f>
+        <v>941.363259838504</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <f aca="false">Revenue_Build!I78</f>
+        <v>1039.56261780077</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <f aca="false">Revenue_Build!J78</f>
+        <v>1129.24274482966</v>
+      </c>
+      <c r="J22" s="12" t="n">
+        <f aca="false">Revenue_Build!K78</f>
+        <v>1205.79455276005</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <f aca="false">Revenue_Build!L78</f>
+        <v>1264.8691601849</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <f aca="false">Revenue_Build!M78</f>
+        <v>1302.81523499045</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="C23" s="12" t="n">
+        <f aca="false">Revenue_Build!D105</f>
+        <v>-7.435</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <f aca="false">Revenue_Build!E105</f>
+        <v>11.5939687444542</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <f aca="false">Revenue_Build!F105</f>
+        <v>31.5380831371095</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <f aca="false">Revenue_Build!G105</f>
+        <v>51.7111115161533</v>
+      </c>
+      <c r="G23" s="12" t="n">
+        <f aca="false">Revenue_Build!H105</f>
+        <v>72.7962689594767</v>
+      </c>
+      <c r="H23" s="12" t="n">
+        <f aca="false">Revenue_Build!I105</f>
+        <v>92.127588212965</v>
+      </c>
+      <c r="I23" s="12" t="n">
+        <f aca="false">Revenue_Build!J105</f>
+        <v>108.556518867661</v>
+      </c>
+      <c r="J23" s="12" t="n">
+        <f aca="false">Revenue_Build!K105</f>
+        <v>120.91787048115</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <f aca="false">Revenue_Build!L105</f>
+        <v>128.116558610273</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <f aca="false">Revenue_Build!M105</f>
+        <v>129.220418985752</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="C24" s="13" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H24" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J24" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K24" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="L24" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M24" s="18" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="C25" s="11" t="n">
+        <f aca="false">C22*C24</f>
+        <v>63.445155</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <f aca="false">D22*D24</f>
+        <v>61.9275390003464</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <f aca="false">E22*E24</f>
+        <v>59.3697983008263</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <f aca="false">F22*F24</f>
+        <v>54.5423774074695</v>
+      </c>
+      <c r="G25" s="11" t="n">
+        <f aca="false">G22*G24</f>
+        <v>47.0681629919252</v>
+      </c>
+      <c r="H25" s="11" t="n">
+        <f aca="false">H22*H24</f>
+        <v>51.9781308900385</v>
+      </c>
+      <c r="I25" s="11" t="n">
+        <f aca="false">I22*I24</f>
+        <v>56.4621372414829</v>
+      </c>
+      <c r="J25" s="11" t="n">
+        <f aca="false">J22*J24</f>
+        <v>60.2897276380024</v>
+      </c>
+      <c r="K25" s="11" t="n">
+        <f aca="false">K22*K24</f>
+        <v>63.2434580092452</v>
+      </c>
+      <c r="L25" s="11" t="n">
+        <f aca="false">L22*L24</f>
+        <v>65.1407617495226</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="C26" s="11" t="n">
+        <f aca="false">C23-$C$15*C25</f>
+        <v>-70.880155</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <f aca="false">D23-$C$15*D25</f>
+        <v>-50.3335702558922</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <f aca="false">E23-$C$15*E25</f>
+        <v>-27.8317151637168</v>
+      </c>
+      <c r="F26" s="11" t="n">
+        <f aca="false">F23-$C$15*F25</f>
+        <v>-2.83126589131614</v>
+      </c>
+      <c r="G26" s="11" t="n">
+        <f aca="false">G23-$C$15*G25</f>
+        <v>25.7281059675515</v>
+      </c>
+      <c r="H26" s="11" t="n">
+        <f aca="false">H23-$C$15*H25</f>
+        <v>40.1494573229264</v>
+      </c>
+      <c r="I26" s="11" t="n">
+        <f aca="false">I23-$C$15*I25</f>
+        <v>52.0943816261782</v>
+      </c>
+      <c r="J26" s="11" t="n">
+        <f aca="false">J23-$C$15*J25</f>
+        <v>60.6281428431472</v>
+      </c>
+      <c r="K26" s="11" t="n">
+        <f aca="false">K23-$C$15*K25</f>
+        <v>64.8731006010278</v>
+      </c>
+      <c r="L26" s="11" t="n">
+        <f aca="false">L23-$C$15*L25</f>
+        <v>64.0796572362299</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <f aca="false">C22*$C$12</f>
+        <v>9.378849</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <f aca="false">D22*$C$12</f>
+        <v>10.9663350313113</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <f aca="false">E22*$C$12</f>
+        <v>12.6160821389256</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <f aca="false">F22*$C$12</f>
+        <v>14.2649294757997</v>
+      </c>
+      <c r="G27" s="11" t="n">
+        <f aca="false">G22*$C$12</f>
+        <v>16.0031754172546</v>
+      </c>
+      <c r="H27" s="11" t="n">
+        <f aca="false">H22*$C$12</f>
+        <v>17.6725645026131</v>
+      </c>
+      <c r="I27" s="11" t="n">
+        <f aca="false">I22*$C$12</f>
+        <v>19.1971266621042</v>
+      </c>
+      <c r="J27" s="11" t="n">
+        <f aca="false">J22*$C$12</f>
+        <v>20.4985073969208</v>
+      </c>
+      <c r="K27" s="11" t="n">
+        <f aca="false">K22*$C$12</f>
+        <v>21.5027757231434</v>
+      </c>
+      <c r="L27" s="11" t="n">
+        <f aca="false">L22*$C$12</f>
+        <v>22.1478589948377</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <f aca="false">C26-C27</f>
+        <v>-80.259004</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <f aca="false">D26-D27</f>
+        <v>-61.2999052872036</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <f aca="false">E26-E27</f>
+        <v>-40.4477973026423</v>
+      </c>
+      <c r="F28" s="11" t="n">
+        <f aca="false">F26-F27</f>
+        <v>-17.0961953671158</v>
+      </c>
+      <c r="G28" s="11" t="n">
+        <f aca="false">G26-G27</f>
+        <v>9.72493055029693</v>
+      </c>
+      <c r="H28" s="11" t="n">
+        <f aca="false">H26-H27</f>
+        <v>22.4768928203134</v>
+      </c>
+      <c r="I28" s="11" t="n">
+        <f aca="false">I26-I27</f>
+        <v>32.897254964074</v>
+      </c>
+      <c r="J28" s="11" t="n">
+        <f aca="false">J26-J27</f>
+        <v>40.1296354462264</v>
+      </c>
+      <c r="K28" s="11" t="n">
+        <f aca="false">K26-K27</f>
+        <v>43.3703248778844</v>
+      </c>
+      <c r="L28" s="11" t="n">
+        <f aca="false">L26-L27</f>
+        <v>41.9317982413922</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="C29" s="11" t="n">
+        <f aca="false">IF(2026&gt;=$C$11,MAX(0,C28)*$C$10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <f aca="false">IF(2027&gt;=$C$11,MAX(0,D28)*$C$10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <f aca="false">IF(2028&gt;=$C$11,MAX(0,E28)*$C$10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="11" t="n">
+        <f aca="false">IF(2029&gt;=$C$11,MAX(0,F28)*$C$10,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="11" t="n">
+        <f aca="false">IF(2030&gt;=$C$11,MAX(0,G28)*$C$10,0)</f>
+        <v>2.43123263757423</v>
+      </c>
+      <c r="H29" s="11" t="n">
+        <f aca="false">IF(2031&gt;=$C$11,MAX(0,H28)*$C$10,0)</f>
+        <v>5.61922320507834</v>
+      </c>
+      <c r="I29" s="11" t="n">
+        <f aca="false">IF(2032&gt;=$C$11,MAX(0,I28)*$C$10,0)</f>
+        <v>8.22431374101851</v>
+      </c>
+      <c r="J29" s="11" t="n">
+        <f aca="false">IF(2033&gt;=$C$11,MAX(0,J28)*$C$10,0)</f>
+        <v>10.0324088615566</v>
+      </c>
+      <c r="K29" s="11" t="n">
+        <f aca="false">IF(2034&gt;=$C$11,MAX(0,K28)*$C$10,0)</f>
+        <v>10.8425812194711</v>
+      </c>
+      <c r="L29" s="11" t="n">
+        <f aca="false">IF(2035&gt;=$C$11,MAX(0,L28)*$C$10,0)</f>
+        <v>10.482949560348</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="C30" s="11" t="n">
+        <f aca="false">C22*$C$13</f>
+        <v>8.275455</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <f aca="false">D22*$C$13</f>
+        <v>9.67617796880412</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <f aca="false">E22*$C$13</f>
+        <v>11.1318371814049</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <f aca="false">F22*$C$13</f>
+        <v>12.5867024786468</v>
+      </c>
+      <c r="G30" s="11" t="n">
+        <f aca="false">G22*$C$13</f>
+        <v>14.1204488975776</v>
+      </c>
+      <c r="H30" s="11" t="n">
+        <f aca="false">H22*$C$13</f>
+        <v>15.5934392670116</v>
+      </c>
+      <c r="I30" s="11" t="n">
+        <f aca="false">I22*$C$13</f>
+        <v>16.9386411724449</v>
+      </c>
+      <c r="J30" s="11" t="n">
+        <f aca="false">J22*$C$13</f>
+        <v>18.0869182914007</v>
+      </c>
+      <c r="K30" s="11" t="n">
+        <f aca="false">K22*$C$13</f>
+        <v>18.9730374027736</v>
+      </c>
+      <c r="L30" s="11" t="n">
+        <f aca="false">L22*$C$13</f>
+        <v>19.5422285248568</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <f aca="false">(D22-C22)*$C$14</f>
+        <v>7.47052250028866</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <f aca="false">(E22-D22)*$C$14</f>
+        <v>7.7635158005376</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <f aca="false">(F22-E22)*$C$14</f>
+        <v>7.75928158528999</v>
+      </c>
+      <c r="G31" s="11" t="n">
+        <f aca="false">(G22-F22)*$C$14</f>
+        <v>8.17998090096409</v>
+      </c>
+      <c r="H31" s="11" t="n">
+        <f aca="false">(H22-G22)*$C$14</f>
+        <v>7.85594863698127</v>
+      </c>
+      <c r="I31" s="11" t="n">
+        <f aca="false">(I22-H22)*$C$14</f>
+        <v>7.17441016231107</v>
+      </c>
+      <c r="J31" s="11" t="n">
+        <f aca="false">(J22-I22)*$C$14</f>
+        <v>6.12414463443121</v>
+      </c>
+      <c r="K31" s="11" t="n">
+        <f aca="false">(K22-J22)*$C$14</f>
+        <v>4.72596859398847</v>
+      </c>
+      <c r="L31" s="11" t="n">
+        <f aca="false">(L22-K22)*$C$14</f>
+        <v>3.03568598444379</v>
+      </c>
+      <c r="M31" s="18" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="16" t="s">
+        <v>558</v>
+      </c>
+      <c r="C32" s="11" t="n">
+        <f aca="false">C26-C29-C30-C31</f>
+        <v>-79.15561</v>
+      </c>
+      <c r="D32" s="11" t="n">
+        <f aca="false">D26-D29-D30-D31</f>
+        <v>-67.480270724985</v>
+      </c>
+      <c r="E32" s="11" t="n">
+        <f aca="false">E26-E29-E30-E31</f>
+        <v>-46.7270681456593</v>
+      </c>
+      <c r="F32" s="11" t="n">
+        <f aca="false">F26-F29-F30-F31</f>
+        <v>-23.1772499552529</v>
+      </c>
+      <c r="G32" s="11" t="n">
+        <f aca="false">G26-G29-G30-G31</f>
+        <v>0.99644353143561</v>
+      </c>
+      <c r="H32" s="11" t="n">
+        <f aca="false">H26-H29-H30-H31</f>
+        <v>11.0808462138553</v>
+      </c>
+      <c r="I32" s="11" t="n">
+        <f aca="false">I26-I29-I30-I31</f>
+        <v>19.7570165504038</v>
+      </c>
+      <c r="J32" s="11" t="n">
+        <f aca="false">J26-J29-J30-J31</f>
+        <v>26.3846710557587</v>
+      </c>
+      <c r="K32" s="11" t="n">
+        <f aca="false">K26-K29-K30-K31</f>
+        <v>30.3315133847946</v>
+      </c>
+      <c r="L32" s="11" t="n">
+        <f aca="false">L26-L29-L30-L31</f>
+        <v>31.0187931665813</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="D33" s="39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E33" s="39" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F33" s="39" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G33" s="39" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H33" s="39" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I33" s="39" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J33" s="39" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="K33" s="39" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="L33" s="39" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <f aca="false">D32/(1+$C$8)^D33</f>
+        <v>-63.9343450905063</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <f aca="false">E32/(1+$C$8)^E33</f>
+        <v>-39.7411789069771</v>
+      </c>
+      <c r="F34" s="11" t="n">
+        <f aca="false">F32/(1+$C$8)^F33</f>
+        <v>-17.6949331949023</v>
+      </c>
+      <c r="G34" s="11" t="n">
+        <f aca="false">G32/(1+$C$8)^G33</f>
+        <v>0.682895929869275</v>
+      </c>
+      <c r="H34" s="11" t="n">
+        <f aca="false">H32/(1+$C$8)^H33</f>
+        <v>6.81694152634891</v>
+      </c>
+      <c r="I34" s="11" t="n">
+        <f aca="false">I32/(1+$C$8)^I33</f>
+        <v>10.9107050106802</v>
+      </c>
+      <c r="J34" s="11" t="n">
+        <f aca="false">J32/(1+$C$8)^J33</f>
+        <v>13.079704838416</v>
+      </c>
+      <c r="K34" s="11" t="n">
+        <f aca="false">K32/(1+$C$8)^K33</f>
+        <v>13.497556329866</v>
+      </c>
+      <c r="L34" s="11" t="n">
+        <f aca="false">L32/(1+$C$8)^L33</f>
+        <v>12.3908407339699</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="3" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="C37" s="11" t="n">
+        <f aca="false">SUM(D34:L34)</f>
+        <v>-63.9918128232354</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <f aca="false">L32*(1+C9)/(C8-C9)</f>
+        <v>380.349487637842</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="C39" s="11" t="n">
+        <f aca="false">C38/(1+C8)^9</f>
+        <v>143.951474596466</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="16" t="s">
+        <v>565</v>
+      </c>
+      <c r="C40" s="11" t="n">
+        <f aca="false">C37+C39</f>
+        <v>79.9596617732309</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <f aca="false">C16</f>
+        <v>336</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="C42" s="11" t="n">
+        <f aca="false">C40+C41</f>
+        <v>415.959661773231</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="16" t="s">
+        <v>568</v>
+      </c>
+      <c r="C43" s="40" t="n">
+        <f aca="false">C42/C17</f>
+        <v>4.94013850086973</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="C44" s="31" t="n">
+        <f aca="false">C43/C18-1</f>
+        <v>-0.825867518474807</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="C45" s="15" t="n">
+        <f aca="false">C39/C40</f>
+        <v>1.80030119442875</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="C47" s="11" t="n">
+        <f aca="false">L23*C19</f>
+        <v>1938.30628478629</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="C48" s="26" t="n">
+        <f aca="false">(C37+C47/(1+C8)^9+C16)/C17</f>
+        <v>11.9430171601853</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="C49" s="15" t="n">
+        <f aca="false">(C47*C8-L32)/(C47+L32)</f>
+        <v>0.0964534120981734</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="3" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="16" t="s">
+        <v>575</v>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D52" s="13" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="13" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C53" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B53)^$D$33:$L$33))+$L$32*(1+C$52)/($B53-C$52)/(1+$B53)^9+$C$16)/$C$17</f>
+        <v>5.7738089304594</v>
+      </c>
+      <c r="D53" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B53)^$D$33:$L$33))+$L$32*(1+D$52)/($B53-D$52)/(1+$B53)^9+$C$16)/$C$17</f>
+        <v>5.97697885980673</v>
+      </c>
+      <c r="E53" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B53)^$D$33:$L$33))+$L$32*(1+E$52)/($B53-E$52)/(1+$B53)^9+$C$16)/$C$17</f>
+        <v>6.21401044404529</v>
+      </c>
+      <c r="F53" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B53)^$D$33:$L$33))+$L$32*(1+F$52)/($B53-F$52)/(1+$B53)^9+$C$16)/$C$17</f>
+        <v>6.49413867996357</v>
+      </c>
+      <c r="G53" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B53)^$D$33:$L$33))+$L$32*(1+G$52)/($B53-G$52)/(1+$B53)^9+$C$16)/$C$17</f>
+        <v>6.83029256306552</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C54" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B54)^$D$33:$L$33))+$L$32*(1+C$52)/($B54-C$52)/(1+$B54)^9+$C$16)/$C$17</f>
+        <v>5.2622948167931</v>
+      </c>
+      <c r="D54" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B54)^$D$33:$L$33))+$L$32*(1+D$52)/($B54-D$52)/(1+$B54)^9+$C$16)/$C$17</f>
+        <v>5.40551033478013</v>
+      </c>
+      <c r="E54" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B54)^$D$33:$L$33))+$L$32*(1+E$52)/($B54-E$52)/(1+$B54)^9+$C$16)/$C$17</f>
+        <v>5.56918521247959</v>
+      </c>
+      <c r="F54" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B54)^$D$33:$L$33))+$L$32*(1+F$52)/($B54-F$52)/(1+$B54)^9+$C$16)/$C$17</f>
+        <v>5.75804084059435</v>
+      </c>
+      <c r="G54" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B54)^$D$33:$L$33))+$L$32*(1+G$52)/($B54-G$52)/(1+$B54)^9+$C$16)/$C$17</f>
+        <v>5.97837240672824</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="13" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="C55" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B55)^$D$33:$L$33))+$L$32*(1+C$52)/($B55-C$52)/(1+$B55)^9+$C$16)/$C$17</f>
+        <v>4.87348623784251</v>
+      </c>
+      <c r="D55" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B55)^$D$33:$L$33))+$L$32*(1+D$52)/($B55-D$52)/(1+$B55)^9+$C$16)/$C$17</f>
+        <v>4.97796729165282</v>
+      </c>
+      <c r="E55" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B55)^$D$33:$L$33))+$L$32*(1+E$52)/($B55-E$52)/(1+$B55)^9+$C$16)/$C$17</f>
+        <v>5.09550847718942</v>
+      </c>
+      <c r="F55" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B55)^$D$33:$L$33))+$L$32*(1+F$52)/($B55-F$52)/(1+$B55)^9+$C$16)/$C$17</f>
+        <v>5.22872182079757</v>
+      </c>
+      <c r="G55" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B55)^$D$33:$L$33))+$L$32*(1+G$52)/($B55-G$52)/(1+$B55)^9+$C$16)/$C$17</f>
+        <v>5.38096564206403</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C56" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B56)^$D$33:$L$33))+$L$32*(1+C$52)/($B56-C$52)/(1+$B56)^9+$C$16)/$C$17</f>
+        <v>4.5700797025027</v>
+      </c>
+      <c r="D56" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B56)^$D$33:$L$33))+$L$32*(1+D$52)/($B56-D$52)/(1+$B56)^9+$C$16)/$C$17</f>
+        <v>4.64838930565399</v>
+      </c>
+      <c r="E56" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B56)^$D$33:$L$33))+$L$32*(1+E$52)/($B56-E$52)/(1+$B56)^9+$C$16)/$C$17</f>
+        <v>4.73539997582209</v>
+      </c>
+      <c r="F56" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B56)^$D$33:$L$33))+$L$32*(1+F$52)/($B56-F$52)/(1+$B56)^9+$C$16)/$C$17</f>
+        <v>4.83264719542173</v>
+      </c>
+      <c r="G56" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B56)^$D$33:$L$33))+$L$32*(1+G$52)/($B56-G$52)/(1+$B56)^9+$C$16)/$C$17</f>
+        <v>4.94205031747133</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="13" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="C57" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B57)^$D$33:$L$33))+$L$32*(1+C$52)/($B57-C$52)/(1+$B57)^9+$C$16)/$C$17</f>
+        <v>4.32837283640384</v>
+      </c>
+      <c r="D57" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B57)^$D$33:$L$33))+$L$32*(1+D$52)/($B57-D$52)/(1+$B57)^9+$C$16)/$C$17</f>
+        <v>4.38836206504073</v>
+      </c>
+      <c r="E57" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B57)^$D$33:$L$33))+$L$32*(1+E$52)/($B57-E$52)/(1+$B57)^9+$C$16)/$C$17</f>
+        <v>4.45435021654131</v>
+      </c>
+      <c r="F57" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B57)^$D$33:$L$33))+$L$32*(1+F$52)/($B57-F$52)/(1+$B57)^9+$C$16)/$C$17</f>
+        <v>4.52728448925247</v>
+      </c>
+      <c r="G57" s="26" t="n">
+        <f aca="false">(SUMPRODUCT($D$32:$L$32/((1+$B57)^$D$33:$L$33))+$L$32*(1+G$52)/($B57-G$52)/(1+$B57)^9+$C$16)/$C$17</f>
+        <v>4.60832257004265</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="18" t="s">
+        <v>576</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:C40"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2520,100 +6681,100 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>430</v>
+        <v>577</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="34" t="s">
-        <v>431</v>
+      <c r="A2" s="41" t="s">
+        <v>578</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>432</v>
+        <v>579</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>433</v>
+        <v>580</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>434</v>
+        <v>581</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>435</v>
+        <v>582</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>436</v>
+        <v>583</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>437</v>
+        <v>584</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>438</v>
+        <v>585</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>439</v>
+        <v>586</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>440</v>
+        <v>587</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>441</v>
+        <v>588</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>442</v>
+        <v>589</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>443</v>
+        <v>590</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>444</v>
+        <v>591</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>445</v>
+        <v>592</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>446</v>
+        <v>593</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>447</v>
+        <v>594</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>448</v>
+        <v>595</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>449</v>
+        <v>596</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>450</v>
+        <v>597</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>451</v>
+        <v>598</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>452</v>
+        <v>599</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>453</v>
+        <v>600</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>454</v>
+        <v>601</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>455</v>
+        <v>602</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2621,43 +6782,43 @@
         <v>231</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>456</v>
+        <v>603</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>457</v>
+        <v>604</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>458</v>
+        <v>605</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>459</v>
+        <v>606</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>460</v>
+        <v>607</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>461</v>
+        <v>608</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>462</v>
+        <v>609</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>463</v>
+        <v>610</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>464</v>
+        <v>611</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>465</v>
+        <v>612</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>466</v>
+        <v>613</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2665,10 +6826,10 @@
         <v>258</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>467</v>
+        <v>614</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>468</v>
+        <v>615</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2676,21 +6837,21 @@
         <v>268</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>469</v>
+        <v>616</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>470</v>
+        <v>617</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>471</v>
+        <v>618</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>472</v>
+        <v>619</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>473</v>
+        <v>620</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2698,10 +6859,10 @@
         <v>262</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>474</v>
+        <v>621</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>475</v>
+        <v>622</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2709,21 +6870,21 @@
         <v>281</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>476</v>
+        <v>623</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>477</v>
+        <v>624</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>478</v>
+        <v>625</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>479</v>
+        <v>626</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>480</v>
+        <v>627</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2731,10 +6892,10 @@
         <v>289</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>481</v>
+        <v>628</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>482</v>
+        <v>629</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2742,10 +6903,10 @@
         <v>294</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>483</v>
+        <v>630</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>484</v>
+        <v>631</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2753,21 +6914,21 @@
         <v>245</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>485</v>
+        <v>632</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>486</v>
+        <v>633</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>487</v>
+        <v>634</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>488</v>
+        <v>635</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>489</v>
+        <v>636</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2775,10 +6936,10 @@
         <v>299</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>490</v>
+        <v>637</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>491</v>
+        <v>638</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2786,21 +6947,21 @@
         <v>221</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>492</v>
+        <v>639</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>493</v>
+        <v>640</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>494</v>
+        <v>641</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>495</v>
+        <v>642</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>496</v>
+        <v>643</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2808,10 +6969,10 @@
         <v>239</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>497</v>
+        <v>644</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>498</v>
+        <v>645</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2819,65 +6980,65 @@
         <v>277</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>499</v>
+        <v>646</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>500</v>
+        <v>647</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>501</v>
+        <v>648</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>502</v>
+        <v>649</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>503</v>
+        <v>650</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>504</v>
+        <v>651</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>505</v>
+        <v>652</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>443</v>
+        <v>590</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>506</v>
+        <v>653</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>507</v>
+        <v>654</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>455</v>
+        <v>602</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>508</v>
+        <v>655</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>509</v>
+        <v>656</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>510</v>
+        <v>657</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>511</v>
+        <v>658</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>512</v>
+        <v>659</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>457</v>
+        <v>604</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2885,38 +7046,38 @@
         <v>254</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>513</v>
+        <v>660</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>480</v>
+        <v>627</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>514</v>
+        <v>661</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>515</v>
+        <v>662</v>
       </c>
       <c r="C37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>516</v>
+        <v>663</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>517</v>
+        <v>664</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>518</v>
+        <v>665</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>519</v>
+        <v>666</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>520</v>
+        <v>667</v>
       </c>
       <c r="C39" s="4"/>
     </row>
@@ -2925,7 +7086,7 @@
         <v>203</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>521</v>
+        <v>668</v>
       </c>
       <c r="C40" s="4"/>
     </row>

</xml_diff>